<commit_message>
Fix database duplication, preserve original Excel columns layout and cleanup users
</commit_message>
<xml_diff>
--- a/training.xlsx
+++ b/training.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\طلاب من اجل مصر\cheating\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8418572E-76A5-45C4-8A07-167889076670}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E3631E6-3A96-4CD6-B9B5-125CE6FAF392}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1555" uniqueCount="914">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1555" uniqueCount="917">
   <si>
     <t>Email Address</t>
   </si>
@@ -2720,9 +2720,6 @@
     <t>01010909308</t>
   </si>
   <si>
-    <t xml:space="preserve">شريف مصطفي عبد المنعم مصطفي </t>
-  </si>
-  <si>
     <t>level 1</t>
   </si>
   <si>
@@ -2756,15 +2753,6 @@
     <t>Student</t>
   </si>
   <si>
-    <t xml:space="preserve">مروان صبحي محمد مصيلحي </t>
-  </si>
-  <si>
-    <t>2023170570@cis.asu.edu.eg</t>
-  </si>
-  <si>
-    <t>01010266849</t>
-  </si>
-  <si>
     <t>Admin</t>
   </si>
   <si>
@@ -2778,6 +2766,27 @@
   </si>
   <si>
     <t>Media</t>
+  </si>
+  <si>
+    <t>2023170714@cis.asu.edu.eg</t>
+  </si>
+  <si>
+    <t>2022170578@cis.asu.edu.eg</t>
+  </si>
+  <si>
+    <t>2023170573@cis.asu.edu.eg</t>
+  </si>
+  <si>
+    <t>01154890597</t>
+  </si>
+  <si>
+    <t>01129324608</t>
+  </si>
+  <si>
+    <t>01113187090</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Level 4 </t>
   </si>
 </sst>
 </file>
@@ -2828,12 +2837,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
@@ -2845,13 +2851,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -3142,14 +3148,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I225"/>
+  <dimension ref="A1:I224"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="33.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="45.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="30.5546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="30.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.6640625" style="7" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="68" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="49.109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.21875" customWidth="1"/>
@@ -3157,7 +3163,7 @@
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>903</v>
+        <v>902</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -3171,7 +3177,7 @@
       <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -3181,7 +3187,7 @@
         <v>6</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>904</v>
+        <v>903</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
@@ -3200,7 +3206,7 @@
       <c r="E2" s="1">
         <v>20251700588</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="6" t="s">
         <v>10</v>
       </c>
       <c r="G2" s="1" t="s">
@@ -3210,7 +3216,7 @@
         <v>12</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
@@ -3229,7 +3235,7 @@
       <c r="E3" s="1">
         <v>20241700031</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="6" t="s">
         <v>16</v>
       </c>
       <c r="G3" s="1" t="s">
@@ -3239,7 +3245,7 @@
         <v>12</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
@@ -3258,7 +3264,7 @@
       <c r="E4" s="1">
         <v>20251700762</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="6" t="s">
         <v>21</v>
       </c>
       <c r="G4" s="1" t="s">
@@ -3268,7 +3274,7 @@
         <v>12</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
@@ -3287,7 +3293,7 @@
       <c r="E5" s="1">
         <v>20251700531</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="6" t="s">
         <v>25</v>
       </c>
       <c r="G5" s="1" t="s">
@@ -3297,7 +3303,7 @@
         <v>12</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
@@ -3316,7 +3322,7 @@
       <c r="E6" s="1">
         <v>2023170451</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="6" t="s">
         <v>29</v>
       </c>
       <c r="G6" s="1" t="s">
@@ -3326,7 +3332,7 @@
         <v>31</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
@@ -3345,7 +3351,7 @@
       <c r="E7" s="1">
         <v>20251700257</v>
       </c>
-      <c r="F7" s="2" t="s">
+      <c r="F7" s="6" t="s">
         <v>35</v>
       </c>
       <c r="G7" s="1" t="s">
@@ -3355,7 +3361,7 @@
         <v>12</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
@@ -3374,7 +3380,7 @@
       <c r="E8" s="1">
         <v>20251700511</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="6" t="s">
         <v>39</v>
       </c>
       <c r="G8" s="1" t="s">
@@ -3384,7 +3390,7 @@
         <v>12</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
@@ -3403,7 +3409,7 @@
       <c r="E9" s="1">
         <v>20251700143</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="6" t="s">
         <v>43</v>
       </c>
       <c r="G9" s="1" t="s">
@@ -3413,7 +3419,7 @@
         <v>12</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
@@ -3432,7 +3438,7 @@
       <c r="E10" s="1">
         <v>20251700720</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="6" t="s">
         <v>47</v>
       </c>
       <c r="G10" s="1" t="s">
@@ -3442,7 +3448,7 @@
         <v>48</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
@@ -3461,7 +3467,7 @@
       <c r="E11" s="1">
         <v>20251700822</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="6" t="s">
         <v>52</v>
       </c>
       <c r="G11" s="1" t="s">
@@ -3471,7 +3477,7 @@
         <v>12</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
@@ -3490,7 +3496,7 @@
       <c r="E12" s="1">
         <v>20241700700</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" s="6" t="s">
         <v>56</v>
       </c>
       <c r="G12" s="1" t="s">
@@ -3500,7 +3506,7 @@
         <v>12</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
@@ -3519,7 +3525,7 @@
       <c r="E13" s="1">
         <v>20241700948</v>
       </c>
-      <c r="F13" s="2" t="s">
+      <c r="F13" s="6" t="s">
         <v>60</v>
       </c>
       <c r="G13" s="1" t="s">
@@ -3529,7 +3535,7 @@
         <v>12</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
@@ -3548,7 +3554,7 @@
       <c r="E14" s="1">
         <v>20251701037</v>
       </c>
-      <c r="F14" s="2" t="s">
+      <c r="F14" s="6" t="s">
         <v>64</v>
       </c>
       <c r="G14" s="1" t="s">
@@ -3558,7 +3564,7 @@
         <v>12</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
@@ -3577,7 +3583,7 @@
       <c r="E15" s="1">
         <v>20251700009</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="F15" s="6" t="s">
         <v>68</v>
       </c>
       <c r="G15" s="1" t="s">
@@ -3587,7 +3593,7 @@
         <v>12</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
@@ -3606,7 +3612,7 @@
       <c r="E16" s="1">
         <v>20241700585</v>
       </c>
-      <c r="F16" s="2" t="s">
+      <c r="F16" s="6" t="s">
         <v>72</v>
       </c>
       <c r="G16" s="1" t="s">
@@ -3616,7 +3622,7 @@
         <v>12</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.3">
@@ -3635,7 +3641,7 @@
       <c r="E17" s="1">
         <v>20241700568</v>
       </c>
-      <c r="F17" s="2" t="s">
+      <c r="F17" s="6" t="s">
         <v>76</v>
       </c>
       <c r="G17" s="1" t="s">
@@ -3645,7 +3651,7 @@
         <v>12</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.3">
@@ -3664,7 +3670,7 @@
       <c r="E18" s="1">
         <v>20241700374</v>
       </c>
-      <c r="F18" s="2" t="s">
+      <c r="F18" s="6" t="s">
         <v>80</v>
       </c>
       <c r="G18" s="1" t="s">
@@ -3674,7 +3680,7 @@
         <v>12</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.3">
@@ -3693,7 +3699,7 @@
       <c r="E19" s="1">
         <v>20251701124</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="F19" s="6" t="s">
         <v>84</v>
       </c>
       <c r="G19" s="1" t="s">
@@ -3703,7 +3709,7 @@
         <v>12</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.3">
@@ -3722,7 +3728,7 @@
       <c r="E20" s="1">
         <v>20241700235</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="F20" s="6" t="s">
         <v>88</v>
       </c>
       <c r="G20" s="1" t="s">
@@ -3732,7 +3738,7 @@
         <v>12</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.3">
@@ -3751,7 +3757,7 @@
       <c r="E21" s="1">
         <v>20241700174</v>
       </c>
-      <c r="F21" s="2" t="s">
+      <c r="F21" s="6" t="s">
         <v>92</v>
       </c>
       <c r="G21" s="1" t="s">
@@ -3761,7 +3767,7 @@
         <v>12</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.3">
@@ -3780,7 +3786,7 @@
       <c r="E22" s="1">
         <v>20241701015</v>
       </c>
-      <c r="F22" s="2" t="s">
+      <c r="F22" s="6" t="s">
         <v>96</v>
       </c>
       <c r="G22" s="1" t="s">
@@ -3790,7 +3796,7 @@
         <v>12</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.3">
@@ -3809,7 +3815,7 @@
       <c r="E23" s="1">
         <v>20241700590</v>
       </c>
-      <c r="F23" s="2" t="s">
+      <c r="F23" s="6" t="s">
         <v>100</v>
       </c>
       <c r="G23" s="1" t="s">
@@ -3819,7 +3825,7 @@
         <v>12</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.3">
@@ -3838,7 +3844,7 @@
       <c r="E24" s="1">
         <v>20241700088</v>
       </c>
-      <c r="F24" s="2" t="s">
+      <c r="F24" s="6" t="s">
         <v>104</v>
       </c>
       <c r="G24" s="1" t="s">
@@ -3848,7 +3854,7 @@
         <v>12</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.3">
@@ -3867,7 +3873,7 @@
       <c r="E25" s="1">
         <v>20241700049</v>
       </c>
-      <c r="F25" s="2" t="s">
+      <c r="F25" s="6" t="s">
         <v>108</v>
       </c>
       <c r="G25" s="1" t="s">
@@ -3877,7 +3883,7 @@
         <v>12</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.3">
@@ -3896,7 +3902,7 @@
       <c r="E26" s="1">
         <v>20251701741</v>
       </c>
-      <c r="F26" s="2" t="s">
+      <c r="F26" s="6" t="s">
         <v>112</v>
       </c>
       <c r="G26" s="1" t="s">
@@ -3906,7 +3912,7 @@
         <v>113</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.3">
@@ -3925,7 +3931,7 @@
       <c r="E27" s="1">
         <v>20241700409</v>
       </c>
-      <c r="F27" s="2" t="s">
+      <c r="F27" s="6" t="s">
         <v>117</v>
       </c>
       <c r="G27" s="1" t="s">
@@ -3935,7 +3941,7 @@
         <v>12</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.3">
@@ -3954,7 +3960,7 @@
       <c r="E28" s="1">
         <v>20241700439</v>
       </c>
-      <c r="F28" s="2" t="s">
+      <c r="F28" s="6" t="s">
         <v>121</v>
       </c>
       <c r="G28" s="1" t="s">
@@ -3964,7 +3970,7 @@
         <v>12</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.3">
@@ -3983,7 +3989,7 @@
       <c r="E29" s="1">
         <v>2023170051</v>
       </c>
-      <c r="F29" s="2" t="s">
+      <c r="F29" s="6" t="s">
         <v>125</v>
       </c>
       <c r="G29" s="1" t="s">
@@ -3993,7 +3999,7 @@
         <v>126</v>
       </c>
       <c r="I29" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.3">
@@ -4012,7 +4018,7 @@
       <c r="E30" s="1">
         <v>20241700232</v>
       </c>
-      <c r="F30" s="2" t="s">
+      <c r="F30" s="6" t="s">
         <v>130</v>
       </c>
       <c r="G30" s="1" t="s">
@@ -4022,7 +4028,7 @@
         <v>12</v>
       </c>
       <c r="I30" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.3">
@@ -4041,7 +4047,7 @@
       <c r="E31" s="1">
         <v>20251700432</v>
       </c>
-      <c r="F31" s="2" t="s">
+      <c r="F31" s="6" t="s">
         <v>134</v>
       </c>
       <c r="G31" s="1" t="s">
@@ -4051,7 +4057,7 @@
         <v>12</v>
       </c>
       <c r="I31" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.3">
@@ -4070,7 +4076,7 @@
       <c r="E32" s="1">
         <v>20241700219</v>
       </c>
-      <c r="F32" s="2" t="s">
+      <c r="F32" s="6" t="s">
         <v>138</v>
       </c>
       <c r="G32" s="1" t="s">
@@ -4080,7 +4086,7 @@
         <v>12</v>
       </c>
       <c r="I32" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.3">
@@ -4099,7 +4105,7 @@
       <c r="E33" s="1">
         <v>2023170020</v>
       </c>
-      <c r="F33" s="2" t="s">
+      <c r="F33" s="6" t="s">
         <v>142</v>
       </c>
       <c r="G33" s="1" t="s">
@@ -4109,7 +4115,7 @@
         <v>31</v>
       </c>
       <c r="I33" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="34" spans="1:9" x14ac:dyDescent="0.3">
@@ -4128,7 +4134,7 @@
       <c r="E34" s="1">
         <v>20251701090</v>
       </c>
-      <c r="F34" s="2" t="s">
+      <c r="F34" s="6" t="s">
         <v>146</v>
       </c>
       <c r="G34" s="1" t="s">
@@ -4138,7 +4144,7 @@
         <v>12</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="35" spans="1:9" x14ac:dyDescent="0.3">
@@ -4157,7 +4163,7 @@
       <c r="E35" s="1">
         <v>2023170533</v>
       </c>
-      <c r="F35" s="2" t="s">
+      <c r="F35" s="6" t="s">
         <v>150</v>
       </c>
       <c r="G35" s="1" t="s">
@@ -4167,7 +4173,7 @@
         <v>31</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.3">
@@ -4186,7 +4192,7 @@
       <c r="E36" s="1">
         <v>2023170218</v>
       </c>
-      <c r="F36" s="2" t="s">
+      <c r="F36" s="6" t="s">
         <v>154</v>
       </c>
       <c r="G36" s="1" t="s">
@@ -4196,7 +4202,7 @@
         <v>31</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.3">
@@ -4215,7 +4221,7 @@
       <c r="E37" s="1">
         <v>2023170036</v>
       </c>
-      <c r="F37" s="2" t="s">
+      <c r="F37" s="6" t="s">
         <v>158</v>
       </c>
       <c r="G37" s="1" t="s">
@@ -4225,7 +4231,7 @@
         <v>126</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.3">
@@ -4244,7 +4250,7 @@
       <c r="E38" s="1">
         <v>20241701017</v>
       </c>
-      <c r="F38" s="2" t="s">
+      <c r="F38" s="6" t="s">
         <v>162</v>
       </c>
       <c r="G38" s="1" t="s">
@@ -4254,7 +4260,7 @@
         <v>12</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.3">
@@ -4273,7 +4279,7 @@
       <c r="E39" s="1">
         <v>2023170213</v>
       </c>
-      <c r="F39" s="2" t="s">
+      <c r="F39" s="6" t="s">
         <v>166</v>
       </c>
       <c r="G39" s="1" t="s">
@@ -4283,7 +4289,7 @@
         <v>48</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.3">
@@ -4302,7 +4308,7 @@
       <c r="E40" s="1">
         <v>2023170731</v>
       </c>
-      <c r="F40" s="2" t="s">
+      <c r="F40" s="6" t="s">
         <v>170</v>
       </c>
       <c r="G40" s="1" t="s">
@@ -4312,7 +4318,7 @@
         <v>31</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.3">
@@ -4331,7 +4337,7 @@
       <c r="E41" s="1">
         <v>20241700600</v>
       </c>
-      <c r="F41" s="2" t="s">
+      <c r="F41" s="6" t="s">
         <v>174</v>
       </c>
       <c r="G41" s="1" t="s">
@@ -4341,7 +4347,7 @@
         <v>12</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.3">
@@ -4360,7 +4366,7 @@
       <c r="E42" s="1">
         <v>2023170356</v>
       </c>
-      <c r="F42" s="2" t="s">
+      <c r="F42" s="6" t="s">
         <v>178</v>
       </c>
       <c r="G42" s="1" t="s">
@@ -4370,7 +4376,7 @@
         <v>31</v>
       </c>
       <c r="I42" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.3">
@@ -4389,7 +4395,7 @@
       <c r="E43" s="1">
         <v>20251700817</v>
       </c>
-      <c r="F43" s="2" t="s">
+      <c r="F43" s="6" t="s">
         <v>182</v>
       </c>
       <c r="G43" s="1" t="s">
@@ -4399,7 +4405,7 @@
         <v>12</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="44" spans="1:9" x14ac:dyDescent="0.3">
@@ -4418,7 +4424,7 @@
       <c r="E44" s="1">
         <v>20241700515</v>
       </c>
-      <c r="F44" s="2" t="s">
+      <c r="F44" s="6" t="s">
         <v>186</v>
       </c>
       <c r="G44" s="1" t="s">
@@ -4428,7 +4434,7 @@
         <v>12</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.3">
@@ -4447,7 +4453,7 @@
       <c r="E45" s="1">
         <v>20241700196</v>
       </c>
-      <c r="F45" s="2" t="s">
+      <c r="F45" s="6" t="s">
         <v>190</v>
       </c>
       <c r="G45" s="1" t="s">
@@ -4457,7 +4463,7 @@
         <v>12</v>
       </c>
       <c r="I45" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.3">
@@ -4476,7 +4482,7 @@
       <c r="E46" s="1">
         <v>20241700528</v>
       </c>
-      <c r="F46" s="2" t="s">
+      <c r="F46" s="6" t="s">
         <v>194</v>
       </c>
       <c r="G46" s="1" t="s">
@@ -4486,7 +4492,7 @@
         <v>12</v>
       </c>
       <c r="I46" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.3">
@@ -4505,7 +4511,7 @@
       <c r="E47" s="1">
         <v>2023170014</v>
       </c>
-      <c r="F47" s="2" t="s">
+      <c r="F47" s="6" t="s">
         <v>198</v>
       </c>
       <c r="G47" s="1" t="s">
@@ -4515,7 +4521,7 @@
         <v>31</v>
       </c>
       <c r="I47" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.3">
@@ -4534,7 +4540,7 @@
       <c r="E48" s="1">
         <v>20251700711</v>
       </c>
-      <c r="F48" s="2" t="s">
+      <c r="F48" s="6" t="s">
         <v>202</v>
       </c>
       <c r="G48" s="1" t="s">
@@ -4544,7 +4550,7 @@
         <v>12</v>
       </c>
       <c r="I48" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.3">
@@ -4563,7 +4569,7 @@
       <c r="E49" s="1">
         <v>20231700227</v>
       </c>
-      <c r="F49" s="2" t="s">
+      <c r="F49" s="6" t="s">
         <v>206</v>
       </c>
       <c r="G49" s="1" t="s">
@@ -4573,7 +4579,7 @@
         <v>207</v>
       </c>
       <c r="I49" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.3">
@@ -4592,7 +4598,7 @@
       <c r="E50" s="1">
         <v>20241700920</v>
       </c>
-      <c r="F50" s="2" t="s">
+      <c r="F50" s="6" t="s">
         <v>211</v>
       </c>
       <c r="G50" s="1" t="s">
@@ -4602,7 +4608,7 @@
         <v>12</v>
       </c>
       <c r="I50" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.3">
@@ -4621,7 +4627,7 @@
       <c r="E51" s="1">
         <v>20251700025</v>
       </c>
-      <c r="F51" s="2" t="s">
+      <c r="F51" s="6" t="s">
         <v>215</v>
       </c>
       <c r="G51" s="1" t="s">
@@ -4631,7 +4637,7 @@
         <v>12</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.3">
@@ -4650,7 +4656,7 @@
       <c r="E52" s="1">
         <v>20241700935</v>
       </c>
-      <c r="F52" s="2" t="s">
+      <c r="F52" s="6" t="s">
         <v>219</v>
       </c>
       <c r="G52" s="1" t="s">
@@ -4660,7 +4666,7 @@
         <v>12</v>
       </c>
       <c r="I52" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.3">
@@ -4679,7 +4685,7 @@
       <c r="E53" s="1">
         <v>2023170326</v>
       </c>
-      <c r="F53" s="2" t="s">
+      <c r="F53" s="6" t="s">
         <v>223</v>
       </c>
       <c r="G53" s="1" t="s">
@@ -4689,7 +4695,7 @@
         <v>31</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.3">
@@ -4708,7 +4714,7 @@
       <c r="E54" s="1">
         <v>20231700213</v>
       </c>
-      <c r="F54" s="2" t="s">
+      <c r="F54" s="6" t="s">
         <v>227</v>
       </c>
       <c r="G54" s="1" t="s">
@@ -4718,7 +4724,7 @@
         <v>207</v>
       </c>
       <c r="I54" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.3">
@@ -4737,7 +4743,7 @@
       <c r="E55" s="1">
         <v>20241700208</v>
       </c>
-      <c r="F55" s="2" t="s">
+      <c r="F55" s="6" t="s">
         <v>231</v>
       </c>
       <c r="G55" s="1" t="s">
@@ -4747,7 +4753,7 @@
         <v>12</v>
       </c>
       <c r="I55" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.3">
@@ -4766,7 +4772,7 @@
       <c r="E56" s="1">
         <v>20231700233</v>
       </c>
-      <c r="F56" s="2" t="s">
+      <c r="F56" s="6" t="s">
         <v>235</v>
       </c>
       <c r="G56" s="1" t="s">
@@ -4776,7 +4782,7 @@
         <v>207</v>
       </c>
       <c r="I56" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.3">
@@ -4795,7 +4801,7 @@
       <c r="E57" s="1">
         <v>2023170065</v>
       </c>
-      <c r="F57" s="2" t="s">
+      <c r="F57" s="6" t="s">
         <v>239</v>
       </c>
       <c r="G57" s="1" t="s">
@@ -4805,7 +4811,7 @@
         <v>31</v>
       </c>
       <c r="I57" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.3">
@@ -4824,7 +4830,7 @@
       <c r="E58" s="1">
         <v>2023170597</v>
       </c>
-      <c r="F58" s="2" t="s">
+      <c r="F58" s="6" t="s">
         <v>243</v>
       </c>
       <c r="G58" s="1" t="s">
@@ -4834,7 +4840,7 @@
         <v>126</v>
       </c>
       <c r="I58" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.3">
@@ -4853,7 +4859,7 @@
       <c r="E59" s="1">
         <v>20241700770</v>
       </c>
-      <c r="F59" s="2" t="s">
+      <c r="F59" s="6" t="s">
         <v>247</v>
       </c>
       <c r="G59" s="1" t="s">
@@ -4863,7 +4869,7 @@
         <v>12</v>
       </c>
       <c r="I59" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.3">
@@ -4882,7 +4888,7 @@
       <c r="E60" s="1">
         <v>20251700271</v>
       </c>
-      <c r="F60" s="2" t="s">
+      <c r="F60" s="6" t="s">
         <v>251</v>
       </c>
       <c r="G60" s="1" t="s">
@@ -4892,7 +4898,7 @@
         <v>12</v>
       </c>
       <c r="I60" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.3">
@@ -4911,7 +4917,7 @@
       <c r="E61" s="1">
         <v>20231700251</v>
       </c>
-      <c r="F61" s="2" t="s">
+      <c r="F61" s="6" t="s">
         <v>255</v>
       </c>
       <c r="G61" s="1" t="s">
@@ -4921,7 +4927,7 @@
         <v>207</v>
       </c>
       <c r="I61" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.3">
@@ -4940,7 +4946,7 @@
       <c r="E62" s="1">
         <v>20241701642</v>
       </c>
-      <c r="F62" s="2" t="s">
+      <c r="F62" s="6" t="s">
         <v>259</v>
       </c>
       <c r="G62" s="1" t="s">
@@ -4950,7 +4956,7 @@
         <v>207</v>
       </c>
       <c r="I62" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="63" spans="1:9" x14ac:dyDescent="0.3">
@@ -4969,7 +4975,7 @@
       <c r="E63" s="1">
         <v>20251700670</v>
       </c>
-      <c r="F63" s="2" t="s">
+      <c r="F63" s="6" t="s">
         <v>263</v>
       </c>
       <c r="G63" s="1" t="s">
@@ -4979,7 +4985,7 @@
         <v>12</v>
       </c>
       <c r="I63" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="64" spans="1:9" x14ac:dyDescent="0.3">
@@ -4998,7 +5004,7 @@
       <c r="E64" s="1">
         <v>20251700575</v>
       </c>
-      <c r="F64" s="2" t="s">
+      <c r="F64" s="6" t="s">
         <v>267</v>
       </c>
       <c r="G64" s="1" t="s">
@@ -5008,7 +5014,7 @@
         <v>12</v>
       </c>
       <c r="I64" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.3">
@@ -5027,7 +5033,7 @@
       <c r="E65" s="1">
         <v>20241700225</v>
       </c>
-      <c r="F65" s="2" t="s">
+      <c r="F65" s="6" t="s">
         <v>271</v>
       </c>
       <c r="G65" s="1" t="s">
@@ -5037,7 +5043,7 @@
         <v>12</v>
       </c>
       <c r="I65" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.3">
@@ -5056,7 +5062,7 @@
       <c r="E66" s="1">
         <v>20251700758</v>
       </c>
-      <c r="F66" s="2" t="s">
+      <c r="F66" s="6" t="s">
         <v>275</v>
       </c>
       <c r="G66" s="1" t="s">
@@ -5066,7 +5072,7 @@
         <v>12</v>
       </c>
       <c r="I66" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.3">
@@ -5085,7 +5091,7 @@
       <c r="E67" s="1">
         <v>20241701603</v>
       </c>
-      <c r="F67" s="2" t="s">
+      <c r="F67" s="6" t="s">
         <v>279</v>
       </c>
       <c r="G67" s="1" t="s">
@@ -5095,7 +5101,7 @@
         <v>207</v>
       </c>
       <c r="I67" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="68" spans="1:9" x14ac:dyDescent="0.3">
@@ -5114,7 +5120,7 @@
       <c r="E68" s="1">
         <v>2023170619</v>
       </c>
-      <c r="F68" s="2" t="s">
+      <c r="F68" s="6" t="s">
         <v>283</v>
       </c>
       <c r="G68" s="1" t="s">
@@ -5124,7 +5130,7 @@
         <v>12</v>
       </c>
       <c r="I68" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.3">
@@ -5143,7 +5149,7 @@
       <c r="E69" s="1">
         <v>20241701909</v>
       </c>
-      <c r="F69" s="2" t="s">
+      <c r="F69" s="6" t="s">
         <v>287</v>
       </c>
       <c r="G69" s="1" t="s">
@@ -5153,7 +5159,7 @@
         <v>288</v>
       </c>
       <c r="I69" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.3">
@@ -5172,7 +5178,7 @@
       <c r="E70" s="1">
         <v>20251700064</v>
       </c>
-      <c r="F70" s="2" t="s">
+      <c r="F70" s="6" t="s">
         <v>292</v>
       </c>
       <c r="G70" s="1" t="s">
@@ -5182,7 +5188,7 @@
         <v>12</v>
       </c>
       <c r="I70" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.3">
@@ -5201,7 +5207,7 @@
       <c r="E71" s="1">
         <v>20251700824</v>
       </c>
-      <c r="F71" s="2" t="s">
+      <c r="F71" s="6" t="s">
         <v>296</v>
       </c>
       <c r="G71" s="1" t="s">
@@ -5211,7 +5217,7 @@
         <v>12</v>
       </c>
       <c r="I71" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.3">
@@ -5230,7 +5236,7 @@
       <c r="E72" s="1">
         <v>20251700770</v>
       </c>
-      <c r="F72" s="2" t="s">
+      <c r="F72" s="6" t="s">
         <v>300</v>
       </c>
       <c r="G72" s="1" t="s">
@@ -5240,7 +5246,7 @@
         <v>12</v>
       </c>
       <c r="I72" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.3">
@@ -5259,7 +5265,7 @@
       <c r="E73" s="1">
         <v>20241701619</v>
       </c>
-      <c r="F73" s="2" t="s">
+      <c r="F73" s="6" t="s">
         <v>304</v>
       </c>
       <c r="G73" s="1" t="s">
@@ -5269,7 +5275,7 @@
         <v>207</v>
       </c>
       <c r="I73" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.3">
@@ -5288,7 +5294,7 @@
       <c r="E74" s="1">
         <v>20251701720</v>
       </c>
-      <c r="F74" s="2" t="s">
+      <c r="F74" s="6" t="s">
         <v>308</v>
       </c>
       <c r="G74" s="1" t="s">
@@ -5298,7 +5304,7 @@
         <v>113</v>
       </c>
       <c r="I74" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="75" spans="1:9" x14ac:dyDescent="0.3">
@@ -5317,7 +5323,7 @@
       <c r="E75" s="1">
         <v>20251700396</v>
       </c>
-      <c r="F75" s="2" t="s">
+      <c r="F75" s="6" t="s">
         <v>312</v>
       </c>
       <c r="G75" s="1" t="s">
@@ -5327,7 +5333,7 @@
         <v>12</v>
       </c>
       <c r="I75" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.3">
@@ -5346,7 +5352,7 @@
       <c r="E76" s="1">
         <v>20251701232</v>
       </c>
-      <c r="F76" s="2" t="s">
+      <c r="F76" s="6" t="s">
         <v>316</v>
       </c>
       <c r="G76" s="1" t="s">
@@ -5356,7 +5362,7 @@
         <v>12</v>
       </c>
       <c r="I76" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="77" spans="1:9" x14ac:dyDescent="0.3">
@@ -5375,7 +5381,7 @@
       <c r="E77" s="1">
         <v>20251701110</v>
       </c>
-      <c r="F77" s="2" t="s">
+      <c r="F77" s="6" t="s">
         <v>320</v>
       </c>
       <c r="G77" s="1" t="s">
@@ -5385,7 +5391,7 @@
         <v>12</v>
       </c>
       <c r="I77" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="78" spans="1:9" x14ac:dyDescent="0.3">
@@ -5404,7 +5410,7 @@
       <c r="E78" s="1">
         <v>20251701070</v>
       </c>
-      <c r="F78" s="2" t="s">
+      <c r="F78" s="6" t="s">
         <v>324</v>
       </c>
       <c r="G78" s="1" t="s">
@@ -5414,7 +5420,7 @@
         <v>12</v>
       </c>
       <c r="I78" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="79" spans="1:9" x14ac:dyDescent="0.3">
@@ -5433,7 +5439,7 @@
       <c r="E79" s="1">
         <v>20251700957</v>
       </c>
-      <c r="F79" s="2" t="s">
+      <c r="F79" s="6" t="s">
         <v>328</v>
       </c>
       <c r="G79" s="1" t="s">
@@ -5443,7 +5449,7 @@
         <v>12</v>
       </c>
       <c r="I79" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="80" spans="1:9" x14ac:dyDescent="0.3">
@@ -5462,7 +5468,7 @@
       <c r="E80" s="1">
         <v>2023170563</v>
       </c>
-      <c r="F80" s="2" t="s">
+      <c r="F80" s="6" t="s">
         <v>332</v>
       </c>
       <c r="G80" s="1" t="s">
@@ -5472,7 +5478,7 @@
         <v>31</v>
       </c>
       <c r="I80" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="81" spans="1:9" x14ac:dyDescent="0.3">
@@ -5491,7 +5497,7 @@
       <c r="E81" s="1">
         <v>2023170720</v>
       </c>
-      <c r="F81" s="2" t="s">
+      <c r="F81" s="6" t="s">
         <v>336</v>
       </c>
       <c r="G81" s="1" t="s">
@@ -5501,7 +5507,7 @@
         <v>31</v>
       </c>
       <c r="I81" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="82" spans="1:9" x14ac:dyDescent="0.3">
@@ -5520,7 +5526,7 @@
       <c r="E82" s="1">
         <v>2025170067</v>
       </c>
-      <c r="F82" s="2" t="s">
+      <c r="F82" s="6" t="s">
         <v>340</v>
       </c>
       <c r="G82" s="1" t="s">
@@ -5530,7 +5536,7 @@
         <v>12</v>
       </c>
       <c r="I82" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.3">
@@ -5549,7 +5555,7 @@
       <c r="E83" s="1">
         <v>2023170530</v>
       </c>
-      <c r="F83" s="2" t="s">
+      <c r="F83" s="6" t="s">
         <v>344</v>
       </c>
       <c r="G83" s="1" t="s">
@@ -5559,7 +5565,7 @@
         <v>31</v>
       </c>
       <c r="I83" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="84" spans="1:9" x14ac:dyDescent="0.3">
@@ -5578,7 +5584,7 @@
       <c r="E84" s="1">
         <v>20251700264</v>
       </c>
-      <c r="F84" s="2" t="s">
+      <c r="F84" s="6" t="s">
         <v>348</v>
       </c>
       <c r="G84" s="1" t="s">
@@ -5588,7 +5594,7 @@
         <v>12</v>
       </c>
       <c r="I84" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="85" spans="1:9" x14ac:dyDescent="0.3">
@@ -5607,7 +5613,7 @@
       <c r="E85" s="1">
         <v>20241700113</v>
       </c>
-      <c r="F85" s="2" t="s">
+      <c r="F85" s="6" t="s">
         <v>352</v>
       </c>
       <c r="G85" s="1" t="s">
@@ -5617,7 +5623,7 @@
         <v>12</v>
       </c>
       <c r="I85" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="86" spans="1:9" x14ac:dyDescent="0.3">
@@ -5636,7 +5642,7 @@
       <c r="E86" s="1">
         <v>20251701116</v>
       </c>
-      <c r="F86" s="2" t="s">
+      <c r="F86" s="6" t="s">
         <v>356</v>
       </c>
       <c r="G86" s="1" t="s">
@@ -5646,7 +5652,7 @@
         <v>12</v>
       </c>
       <c r="I86" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="87" spans="1:9" x14ac:dyDescent="0.3">
@@ -5665,7 +5671,7 @@
       <c r="E87" s="1">
         <v>2023170572</v>
       </c>
-      <c r="F87" s="2" t="s">
+      <c r="F87" s="6" t="s">
         <v>360</v>
       </c>
       <c r="G87" s="1" t="s">
@@ -5675,7 +5681,7 @@
         <v>48</v>
       </c>
       <c r="I87" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="88" spans="1:9" x14ac:dyDescent="0.3">
@@ -5694,7 +5700,7 @@
       <c r="E88" s="1">
         <v>20251700832</v>
       </c>
-      <c r="F88" s="2" t="s">
+      <c r="F88" s="6" t="s">
         <v>364</v>
       </c>
       <c r="G88" s="1" t="s">
@@ -5704,7 +5710,7 @@
         <v>12</v>
       </c>
       <c r="I88" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.3">
@@ -5723,7 +5729,7 @@
       <c r="E89" s="1">
         <v>20241700167</v>
       </c>
-      <c r="F89" s="2" t="s">
+      <c r="F89" s="6" t="s">
         <v>368</v>
       </c>
       <c r="G89" s="1" t="s">
@@ -5733,7 +5739,7 @@
         <v>12</v>
       </c>
       <c r="I89" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="90" spans="1:9" x14ac:dyDescent="0.3">
@@ -5752,7 +5758,7 @@
       <c r="E90" s="1">
         <v>20241701096</v>
       </c>
-      <c r="F90" s="2" t="s">
+      <c r="F90" s="6" t="s">
         <v>372</v>
       </c>
       <c r="G90" s="1" t="s">
@@ -5762,7 +5768,7 @@
         <v>12</v>
       </c>
       <c r="I90" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="91" spans="1:9" x14ac:dyDescent="0.3">
@@ -5781,7 +5787,7 @@
       <c r="E91" s="1">
         <v>2022170197</v>
       </c>
-      <c r="F91" s="2" t="s">
+      <c r="F91" s="6" t="s">
         <v>376</v>
       </c>
       <c r="G91" s="1" t="s">
@@ -5791,7 +5797,7 @@
         <v>377</v>
       </c>
       <c r="I91" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="92" spans="1:9" x14ac:dyDescent="0.3">
@@ -5810,7 +5816,7 @@
       <c r="E92" s="1">
         <v>2023170667</v>
       </c>
-      <c r="F92" s="2" t="s">
+      <c r="F92" s="6" t="s">
         <v>381</v>
       </c>
       <c r="G92" s="1" t="s">
@@ -5820,7 +5826,7 @@
         <v>377</v>
       </c>
       <c r="I92" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="93" spans="1:9" x14ac:dyDescent="0.3">
@@ -5839,7 +5845,7 @@
       <c r="E93" s="1">
         <v>20251700516</v>
       </c>
-      <c r="F93" s="2" t="s">
+      <c r="F93" s="6" t="s">
         <v>385</v>
       </c>
       <c r="G93" s="1" t="s">
@@ -5849,7 +5855,7 @@
         <v>12</v>
       </c>
       <c r="I93" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="94" spans="1:9" x14ac:dyDescent="0.3">
@@ -5868,7 +5874,7 @@
       <c r="E94" s="1">
         <v>20241700510</v>
       </c>
-      <c r="F94" s="2" t="s">
+      <c r="F94" s="6" t="s">
         <v>389</v>
       </c>
       <c r="G94" s="1" t="s">
@@ -5878,7 +5884,7 @@
         <v>12</v>
       </c>
       <c r="I94" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="95" spans="1:9" x14ac:dyDescent="0.3">
@@ -5897,7 +5903,7 @@
       <c r="E95" s="1">
         <v>20251700862</v>
       </c>
-      <c r="F95" s="2" t="s">
+      <c r="F95" s="6" t="s">
         <v>393</v>
       </c>
       <c r="G95" s="1" t="s">
@@ -5907,7 +5913,7 @@
         <v>12</v>
       </c>
       <c r="I95" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="96" spans="1:9" x14ac:dyDescent="0.3">
@@ -5926,7 +5932,7 @@
       <c r="E96" s="1">
         <v>20251700019</v>
       </c>
-      <c r="F96" s="2" t="s">
+      <c r="F96" s="6" t="s">
         <v>397</v>
       </c>
       <c r="G96" s="1" t="s">
@@ -5936,7 +5942,7 @@
         <v>12</v>
       </c>
       <c r="I96" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="97" spans="1:9" x14ac:dyDescent="0.3">
@@ -5955,7 +5961,7 @@
       <c r="E97" s="1">
         <v>20241701556</v>
       </c>
-      <c r="F97" s="2" t="s">
+      <c r="F97" s="6" t="s">
         <v>401</v>
       </c>
       <c r="G97" s="1" t="s">
@@ -5965,7 +5971,7 @@
         <v>402</v>
       </c>
       <c r="I97" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.3">
@@ -5984,7 +5990,7 @@
       <c r="E98" s="1">
         <v>20251700235</v>
       </c>
-      <c r="F98" s="2" t="s">
+      <c r="F98" s="6" t="s">
         <v>406</v>
       </c>
       <c r="G98" s="1" t="s">
@@ -5994,7 +6000,7 @@
         <v>12</v>
       </c>
       <c r="I98" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.3">
@@ -6013,7 +6019,7 @@
       <c r="E99" s="1">
         <v>2023170240</v>
       </c>
-      <c r="F99" s="2" t="s">
+      <c r="F99" s="6" t="s">
         <v>410</v>
       </c>
       <c r="G99" s="1" t="s">
@@ -6023,7 +6029,7 @@
         <v>31</v>
       </c>
       <c r="I99" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.3">
@@ -6042,7 +6048,7 @@
       <c r="E100" s="1">
         <v>20251700564</v>
       </c>
-      <c r="F100" s="2" t="s">
+      <c r="F100" s="6" t="s">
         <v>414</v>
       </c>
       <c r="G100" s="1" t="s">
@@ -6052,7 +6058,7 @@
         <v>12</v>
       </c>
       <c r="I100" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.3">
@@ -6071,7 +6077,7 @@
       <c r="E101" s="1">
         <v>20251700859</v>
       </c>
-      <c r="F101" s="2" t="s">
+      <c r="F101" s="6" t="s">
         <v>418</v>
       </c>
       <c r="G101" s="1" t="s">
@@ -6081,7 +6087,7 @@
         <v>12</v>
       </c>
       <c r="I101" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="102" spans="1:9" x14ac:dyDescent="0.3">
@@ -6100,7 +6106,7 @@
       <c r="E102" s="1">
         <v>20251700704</v>
       </c>
-      <c r="F102" s="2" t="s">
+      <c r="F102" s="6" t="s">
         <v>422</v>
       </c>
       <c r="G102" s="1" t="s">
@@ -6110,7 +6116,7 @@
         <v>12</v>
       </c>
       <c r="I102" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="103" spans="1:9" x14ac:dyDescent="0.3">
@@ -6129,7 +6135,7 @@
       <c r="E103" s="1">
         <v>20251700104</v>
       </c>
-      <c r="F103" s="2" t="s">
+      <c r="F103" s="6" t="s">
         <v>426</v>
       </c>
       <c r="G103" s="1" t="s">
@@ -6139,7 +6145,7 @@
         <v>12</v>
       </c>
       <c r="I103" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.3">
@@ -6158,7 +6164,7 @@
       <c r="E104" s="1">
         <v>20241700924</v>
       </c>
-      <c r="F104" s="2" t="s">
+      <c r="F104" s="6" t="s">
         <v>430</v>
       </c>
       <c r="G104" s="1" t="s">
@@ -6168,7 +6174,7 @@
         <v>12</v>
       </c>
       <c r="I104" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="105" spans="1:9" x14ac:dyDescent="0.3">
@@ -6187,7 +6193,7 @@
       <c r="E105" s="1">
         <v>2023170234</v>
       </c>
-      <c r="F105" s="2" t="s">
+      <c r="F105" s="6" t="s">
         <v>434</v>
       </c>
       <c r="G105" s="1" t="s">
@@ -6197,7 +6203,7 @@
         <v>31</v>
       </c>
       <c r="I105" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="106" spans="1:9" x14ac:dyDescent="0.3">
@@ -6216,7 +6222,7 @@
       <c r="E106" s="1">
         <v>20251700960</v>
       </c>
-      <c r="F106" s="2" t="s">
+      <c r="F106" s="6" t="s">
         <v>438</v>
       </c>
       <c r="G106" s="1" t="s">
@@ -6226,7 +6232,7 @@
         <v>12</v>
       </c>
       <c r="I106" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="107" spans="1:9" x14ac:dyDescent="0.3">
@@ -6245,7 +6251,7 @@
       <c r="E107" s="1">
         <v>20251700500</v>
       </c>
-      <c r="F107" s="2" t="s">
+      <c r="F107" s="6" t="s">
         <v>442</v>
       </c>
       <c r="G107" s="1" t="s">
@@ -6255,7 +6261,7 @@
         <v>12</v>
       </c>
       <c r="I107" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="108" spans="1:9" x14ac:dyDescent="0.3">
@@ -6274,7 +6280,7 @@
       <c r="E108" s="1">
         <v>2023170058</v>
       </c>
-      <c r="F108" s="2" t="s">
+      <c r="F108" s="6" t="s">
         <v>446</v>
       </c>
       <c r="G108" s="1" t="s">
@@ -6284,7 +6290,7 @@
         <v>31</v>
       </c>
       <c r="I108" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="109" spans="1:9" x14ac:dyDescent="0.3">
@@ -6303,7 +6309,7 @@
       <c r="E109" s="1">
         <v>2023170223</v>
       </c>
-      <c r="F109" s="2" t="s">
+      <c r="F109" s="6" t="s">
         <v>450</v>
       </c>
       <c r="G109" s="1" t="s">
@@ -6313,7 +6319,7 @@
         <v>48</v>
       </c>
       <c r="I109" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="110" spans="1:9" x14ac:dyDescent="0.3">
@@ -6332,7 +6338,7 @@
       <c r="E110" s="1">
         <v>20241700341</v>
       </c>
-      <c r="F110" s="2" t="s">
+      <c r="F110" s="6" t="s">
         <v>454</v>
       </c>
       <c r="G110" s="1" t="s">
@@ -6342,7 +6348,7 @@
         <v>12</v>
       </c>
       <c r="I110" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="111" spans="1:9" x14ac:dyDescent="0.3">
@@ -6361,7 +6367,7 @@
       <c r="E111" s="1">
         <v>20251700769</v>
       </c>
-      <c r="F111" s="2" t="s">
+      <c r="F111" s="6" t="s">
         <v>458</v>
       </c>
       <c r="G111" s="1" t="s">
@@ -6371,7 +6377,7 @@
         <v>12</v>
       </c>
       <c r="I111" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="112" spans="1:9" x14ac:dyDescent="0.3">
@@ -6390,7 +6396,7 @@
       <c r="E112" s="1">
         <v>20251701155</v>
       </c>
-      <c r="F112" s="2" t="s">
+      <c r="F112" s="6" t="s">
         <v>462</v>
       </c>
       <c r="G112" s="1" t="s">
@@ -6400,7 +6406,7 @@
         <v>12</v>
       </c>
       <c r="I112" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="113" spans="1:9" x14ac:dyDescent="0.3">
@@ -6419,7 +6425,7 @@
       <c r="E113" s="1">
         <v>20241700943</v>
       </c>
-      <c r="F113" s="2" t="s">
+      <c r="F113" s="6" t="s">
         <v>466</v>
       </c>
       <c r="G113" s="1" t="s">
@@ -6429,7 +6435,7 @@
         <v>12</v>
       </c>
       <c r="I113" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="114" spans="1:9" x14ac:dyDescent="0.3">
@@ -6448,7 +6454,7 @@
       <c r="E114" s="1">
         <v>2023170212</v>
       </c>
-      <c r="F114" s="2" t="s">
+      <c r="F114" s="6" t="s">
         <v>470</v>
       </c>
       <c r="G114" s="1" t="s">
@@ -6458,7 +6464,7 @@
         <v>31</v>
       </c>
       <c r="I114" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="115" spans="1:9" x14ac:dyDescent="0.3">
@@ -6477,7 +6483,7 @@
       <c r="E115" s="1">
         <v>20241701169</v>
       </c>
-      <c r="F115" s="2" t="s">
+      <c r="F115" s="6" t="s">
         <v>474</v>
       </c>
       <c r="G115" s="1" t="s">
@@ -6487,7 +6493,7 @@
         <v>12</v>
       </c>
       <c r="I115" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="116" spans="1:9" x14ac:dyDescent="0.3">
@@ -6506,7 +6512,7 @@
       <c r="E116" s="1">
         <v>20241700794</v>
       </c>
-      <c r="F116" s="2" t="s">
+      <c r="F116" s="6" t="s">
         <v>478</v>
       </c>
       <c r="G116" s="1" t="s">
@@ -6516,7 +6522,7 @@
         <v>12</v>
       </c>
       <c r="I116" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="117" spans="1:9" x14ac:dyDescent="0.3">
@@ -6535,7 +6541,7 @@
       <c r="E117" s="1">
         <v>20251700666</v>
       </c>
-      <c r="F117" s="2" t="s">
+      <c r="F117" s="6" t="s">
         <v>482</v>
       </c>
       <c r="G117" s="1" t="s">
@@ -6545,7 +6551,7 @@
         <v>12</v>
       </c>
       <c r="I117" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="118" spans="1:9" x14ac:dyDescent="0.3">
@@ -6564,7 +6570,7 @@
       <c r="E118" s="1">
         <v>2023170466</v>
       </c>
-      <c r="F118" s="2" t="s">
+      <c r="F118" s="6" t="s">
         <v>486</v>
       </c>
       <c r="G118" s="1" t="s">
@@ -6574,7 +6580,7 @@
         <v>31</v>
       </c>
       <c r="I118" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="119" spans="1:9" x14ac:dyDescent="0.3">
@@ -6593,7 +6599,7 @@
       <c r="E119" s="1">
         <v>20251700750</v>
       </c>
-      <c r="F119" s="2" t="s">
+      <c r="F119" s="6" t="s">
         <v>490</v>
       </c>
       <c r="G119" s="1" t="s">
@@ -6603,7 +6609,7 @@
         <v>12</v>
       </c>
       <c r="I119" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="120" spans="1:9" x14ac:dyDescent="0.3">
@@ -6622,7 +6628,7 @@
       <c r="E120" s="1">
         <v>20251701610</v>
       </c>
-      <c r="F120" s="2" t="s">
+      <c r="F120" s="6" t="s">
         <v>494</v>
       </c>
       <c r="G120" s="1" t="s">
@@ -6632,7 +6638,7 @@
         <v>207</v>
       </c>
       <c r="I120" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="121" spans="1:9" x14ac:dyDescent="0.3">
@@ -6651,7 +6657,7 @@
       <c r="E121" s="1">
         <v>20241700163</v>
       </c>
-      <c r="F121" s="2" t="s">
+      <c r="F121" s="6" t="s">
         <v>498</v>
       </c>
       <c r="G121" s="1" t="s">
@@ -6661,7 +6667,7 @@
         <v>12</v>
       </c>
       <c r="I121" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="122" spans="1:9" x14ac:dyDescent="0.3">
@@ -6680,7 +6686,7 @@
       <c r="E122" s="1">
         <v>20241700631</v>
       </c>
-      <c r="F122" s="2" t="s">
+      <c r="F122" s="6" t="s">
         <v>502</v>
       </c>
       <c r="G122" s="1" t="s">
@@ -6690,7 +6696,7 @@
         <v>12</v>
       </c>
       <c r="I122" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="123" spans="1:9" x14ac:dyDescent="0.3">
@@ -6709,7 +6715,7 @@
       <c r="E123" s="1">
         <v>20251701542</v>
       </c>
-      <c r="F123" s="2" t="s">
+      <c r="F123" s="6" t="s">
         <v>506</v>
       </c>
       <c r="G123" s="1" t="s">
@@ -6719,7 +6725,7 @@
         <v>507</v>
       </c>
       <c r="I123" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="124" spans="1:9" x14ac:dyDescent="0.3">
@@ -6738,7 +6744,7 @@
       <c r="E124" s="1">
         <v>20251700328</v>
       </c>
-      <c r="F124" s="2" t="s">
+      <c r="F124" s="6" t="s">
         <v>511</v>
       </c>
       <c r="G124" s="1" t="s">
@@ -6748,7 +6754,7 @@
         <v>12</v>
       </c>
       <c r="I124" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="125" spans="1:9" x14ac:dyDescent="0.3">
@@ -6767,7 +6773,7 @@
       <c r="E125" s="1">
         <v>20231700255</v>
       </c>
-      <c r="F125" s="2" t="s">
+      <c r="F125" s="6" t="s">
         <v>515</v>
       </c>
       <c r="G125" s="1" t="s">
@@ -6777,7 +6783,7 @@
         <v>207</v>
       </c>
       <c r="I125" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="126" spans="1:9" x14ac:dyDescent="0.3">
@@ -6796,7 +6802,7 @@
       <c r="E126" s="1">
         <v>2023170249</v>
       </c>
-      <c r="F126" s="2" t="s">
+      <c r="F126" s="6" t="s">
         <v>519</v>
       </c>
       <c r="G126" s="1" t="s">
@@ -6806,7 +6812,7 @@
         <v>126</v>
       </c>
       <c r="I126" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="127" spans="1:9" x14ac:dyDescent="0.3">
@@ -6825,7 +6831,7 @@
       <c r="E127" s="1">
         <v>2022170632</v>
       </c>
-      <c r="F127" s="2" t="s">
+      <c r="F127" s="6" t="s">
         <v>523</v>
       </c>
       <c r="G127" s="1" t="s">
@@ -6835,7 +6841,7 @@
         <v>126</v>
       </c>
       <c r="I127" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="128" spans="1:9" x14ac:dyDescent="0.3">
@@ -6854,7 +6860,7 @@
       <c r="E128" s="1">
         <v>2023170302</v>
       </c>
-      <c r="F128" s="2" t="s">
+      <c r="F128" s="6" t="s">
         <v>527</v>
       </c>
       <c r="G128" s="1" t="s">
@@ -6864,7 +6870,7 @@
         <v>126</v>
       </c>
       <c r="I128" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="129" spans="1:9" x14ac:dyDescent="0.3">
@@ -6883,7 +6889,7 @@
       <c r="E129" s="1">
         <v>20241700244</v>
       </c>
-      <c r="F129" s="2" t="s">
+      <c r="F129" s="6" t="s">
         <v>531</v>
       </c>
       <c r="G129" s="1" t="s">
@@ -6893,7 +6899,7 @@
         <v>12</v>
       </c>
       <c r="I129" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.3">
@@ -6912,7 +6918,7 @@
       <c r="E130" s="1">
         <v>2023170417</v>
       </c>
-      <c r="F130" s="2" t="s">
+      <c r="F130" s="6" t="s">
         <v>535</v>
       </c>
       <c r="G130" s="1" t="s">
@@ -6922,7 +6928,7 @@
         <v>126</v>
       </c>
       <c r="I130" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.3">
@@ -6941,7 +6947,7 @@
       <c r="E131" s="1">
         <v>20241701016</v>
       </c>
-      <c r="F131" s="2" t="s">
+      <c r="F131" s="6" t="s">
         <v>539</v>
       </c>
       <c r="G131" s="1" t="s">
@@ -6951,7 +6957,7 @@
         <v>12</v>
       </c>
       <c r="I131" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="132" spans="1:9" x14ac:dyDescent="0.3">
@@ -6970,7 +6976,7 @@
       <c r="E132" s="1">
         <v>20251701012</v>
       </c>
-      <c r="F132" s="2" t="s">
+      <c r="F132" s="6" t="s">
         <v>543</v>
       </c>
       <c r="G132" s="1" t="s">
@@ -6980,7 +6986,7 @@
         <v>12</v>
       </c>
       <c r="I132" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="133" spans="1:9" x14ac:dyDescent="0.3">
@@ -6999,7 +7005,7 @@
       <c r="E133" s="1">
         <v>2023170147</v>
       </c>
-      <c r="F133" s="2" t="s">
+      <c r="F133" s="6" t="s">
         <v>547</v>
       </c>
       <c r="G133" s="1" t="s">
@@ -7009,7 +7015,7 @@
         <v>126</v>
       </c>
       <c r="I133" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="134" spans="1:9" x14ac:dyDescent="0.3">
@@ -7028,7 +7034,7 @@
       <c r="E134" s="1">
         <v>20251700250</v>
       </c>
-      <c r="F134" s="2" t="s">
+      <c r="F134" s="6" t="s">
         <v>551</v>
       </c>
       <c r="G134" s="1" t="s">
@@ -7038,7 +7044,7 @@
         <v>12</v>
       </c>
       <c r="I134" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="135" spans="1:9" x14ac:dyDescent="0.3">
@@ -7057,7 +7063,7 @@
       <c r="E135" s="1">
         <v>20241701056</v>
       </c>
-      <c r="F135" s="2" t="s">
+      <c r="F135" s="6" t="s">
         <v>555</v>
       </c>
       <c r="G135" s="1" t="s">
@@ -7067,7 +7073,7 @@
         <v>12</v>
       </c>
       <c r="I135" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.3">
@@ -7086,7 +7092,7 @@
       <c r="E136" s="1">
         <v>20251700097</v>
       </c>
-      <c r="F136" s="2" t="s">
+      <c r="F136" s="6" t="s">
         <v>559</v>
       </c>
       <c r="G136" s="1" t="s">
@@ -7096,7 +7102,7 @@
         <v>12</v>
       </c>
       <c r="I136" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.3">
@@ -7115,7 +7121,7 @@
       <c r="E137" s="1">
         <v>20251701172</v>
       </c>
-      <c r="F137" s="2" t="s">
+      <c r="F137" s="6" t="s">
         <v>563</v>
       </c>
       <c r="G137" s="1" t="s">
@@ -7125,7 +7131,7 @@
         <v>12</v>
       </c>
       <c r="I137" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.3">
@@ -7144,7 +7150,7 @@
       <c r="E138" s="1">
         <v>2022170068</v>
       </c>
-      <c r="F138" s="2" t="s">
+      <c r="F138" s="6" t="s">
         <v>567</v>
       </c>
       <c r="G138" s="1" t="s">
@@ -7154,7 +7160,7 @@
         <v>48</v>
       </c>
       <c r="I138" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.3">
@@ -7173,7 +7179,7 @@
       <c r="E139" s="1">
         <v>20241700155</v>
       </c>
-      <c r="F139" s="2" t="s">
+      <c r="F139" s="6" t="s">
         <v>572</v>
       </c>
       <c r="G139" s="1" t="s">
@@ -7183,7 +7189,7 @@
         <v>12</v>
       </c>
       <c r="I139" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.3">
@@ -7202,7 +7208,7 @@
       <c r="E140" s="1">
         <v>20251700521</v>
       </c>
-      <c r="F140" s="2" t="s">
+      <c r="F140" s="6" t="s">
         <v>576</v>
       </c>
       <c r="G140" s="1" t="s">
@@ -7212,7 +7218,7 @@
         <v>12</v>
       </c>
       <c r="I140" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.3">
@@ -7231,7 +7237,7 @@
       <c r="E141" s="1">
         <v>20241700953</v>
       </c>
-      <c r="F141" s="2" t="s">
+      <c r="F141" s="6" t="s">
         <v>580</v>
       </c>
       <c r="G141" s="1" t="s">
@@ -7241,7 +7247,7 @@
         <v>12</v>
       </c>
       <c r="I141" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="142" spans="1:9" x14ac:dyDescent="0.3">
@@ -7260,7 +7266,7 @@
       <c r="E142" s="1">
         <v>2018170229</v>
       </c>
-      <c r="F142" s="2" t="s">
+      <c r="F142" s="6" t="s">
         <v>584</v>
       </c>
       <c r="G142" s="1" t="s">
@@ -7270,7 +7276,7 @@
         <v>126</v>
       </c>
       <c r="I142" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="143" spans="1:9" x14ac:dyDescent="0.3">
@@ -7289,7 +7295,7 @@
       <c r="E143" s="1">
         <v>20241700047</v>
       </c>
-      <c r="F143" s="2" t="s">
+      <c r="F143" s="6" t="s">
         <v>588</v>
       </c>
       <c r="G143" s="1" t="s">
@@ -7299,7 +7305,7 @@
         <v>12</v>
       </c>
       <c r="I143" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="144" spans="1:9" x14ac:dyDescent="0.3">
@@ -7318,7 +7324,7 @@
       <c r="E144" s="1">
         <v>20241700089</v>
       </c>
-      <c r="F144" s="2" t="s">
+      <c r="F144" s="6" t="s">
         <v>592</v>
       </c>
       <c r="G144" s="1" t="s">
@@ -7328,7 +7334,7 @@
         <v>12</v>
       </c>
       <c r="I144" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="145" spans="1:9" x14ac:dyDescent="0.3">
@@ -7347,7 +7353,7 @@
       <c r="E145" s="1">
         <v>2023170149</v>
       </c>
-      <c r="F145" s="2" t="s">
+      <c r="F145" s="6" t="s">
         <v>596</v>
       </c>
       <c r="G145" s="1" t="s">
@@ -7357,7 +7363,7 @@
         <v>126</v>
       </c>
       <c r="I145" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="146" spans="1:9" x14ac:dyDescent="0.3">
@@ -7376,7 +7382,7 @@
       <c r="E146" s="1">
         <v>20241700742</v>
       </c>
-      <c r="F146" s="2" t="s">
+      <c r="F146" s="6" t="s">
         <v>600</v>
       </c>
       <c r="G146" s="1" t="s">
@@ -7386,7 +7392,7 @@
         <v>12</v>
       </c>
       <c r="I146" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="147" spans="1:9" x14ac:dyDescent="0.3">
@@ -7405,7 +7411,7 @@
       <c r="E147" s="1">
         <v>20241700036</v>
       </c>
-      <c r="F147" s="2" t="s">
+      <c r="F147" s="6" t="s">
         <v>604</v>
       </c>
       <c r="G147" s="1" t="s">
@@ -7415,7 +7421,7 @@
         <v>12</v>
       </c>
       <c r="I147" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="148" spans="1:9" x14ac:dyDescent="0.3">
@@ -7434,7 +7440,7 @@
       <c r="E148" s="1">
         <v>20251700202</v>
       </c>
-      <c r="F148" s="2" t="s">
+      <c r="F148" s="6" t="s">
         <v>608</v>
       </c>
       <c r="G148" s="1" t="s">
@@ -7444,7 +7450,7 @@
         <v>12</v>
       </c>
       <c r="I148" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="149" spans="1:9" x14ac:dyDescent="0.3">
@@ -7463,7 +7469,7 @@
       <c r="E149" s="1">
         <v>20251700277</v>
       </c>
-      <c r="F149" s="2" t="s">
+      <c r="F149" s="6" t="s">
         <v>612</v>
       </c>
       <c r="G149" s="1" t="s">
@@ -7473,7 +7479,7 @@
         <v>12</v>
       </c>
       <c r="I149" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="150" spans="1:9" x14ac:dyDescent="0.3">
@@ -7492,7 +7498,7 @@
       <c r="E150" s="1">
         <v>2023170364</v>
       </c>
-      <c r="F150" s="2" t="s">
+      <c r="F150" s="6" t="s">
         <v>616</v>
       </c>
       <c r="G150" s="1" t="s">
@@ -7502,7 +7508,7 @@
         <v>31</v>
       </c>
       <c r="I150" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="151" spans="1:9" x14ac:dyDescent="0.3">
@@ -7521,7 +7527,7 @@
       <c r="E151" s="1">
         <v>20251700797</v>
       </c>
-      <c r="F151" s="2" t="s">
+      <c r="F151" s="6" t="s">
         <v>620</v>
       </c>
       <c r="G151" s="1" t="s">
@@ -7531,7 +7537,7 @@
         <v>12</v>
       </c>
       <c r="I151" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="152" spans="1:9" x14ac:dyDescent="0.3">
@@ -7550,7 +7556,7 @@
       <c r="E152" s="1">
         <v>2023170553</v>
       </c>
-      <c r="F152" s="2" t="s">
+      <c r="F152" s="6" t="s">
         <v>624</v>
       </c>
       <c r="G152" s="1" t="s">
@@ -7560,7 +7566,7 @@
         <v>377</v>
       </c>
       <c r="I152" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="153" spans="1:9" x14ac:dyDescent="0.3">
@@ -7579,7 +7585,7 @@
       <c r="E153" s="1">
         <v>2023170495</v>
       </c>
-      <c r="F153" s="2" t="s">
+      <c r="F153" s="6" t="s">
         <v>628</v>
       </c>
       <c r="G153" s="1" t="s">
@@ -7589,7 +7595,7 @@
         <v>12</v>
       </c>
       <c r="I153" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="154" spans="1:9" x14ac:dyDescent="0.3">
@@ -7608,7 +7614,7 @@
       <c r="E154" s="1">
         <v>20251701801</v>
       </c>
-      <c r="F154" s="2" t="s">
+      <c r="F154" s="6" t="s">
         <v>632</v>
       </c>
       <c r="G154" s="1" t="s">
@@ -7618,7 +7624,7 @@
         <v>633</v>
       </c>
       <c r="I154" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="155" spans="1:9" x14ac:dyDescent="0.3">
@@ -7637,7 +7643,7 @@
       <c r="E155" s="1">
         <v>20241700037</v>
       </c>
-      <c r="F155" s="2" t="s">
+      <c r="F155" s="6" t="s">
         <v>637</v>
       </c>
       <c r="G155" s="1" t="s">
@@ -7647,7 +7653,7 @@
         <v>12</v>
       </c>
       <c r="I155" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="156" spans="1:9" x14ac:dyDescent="0.3">
@@ -7666,7 +7672,7 @@
       <c r="E156" s="1">
         <v>20241700044</v>
       </c>
-      <c r="F156" s="2" t="s">
+      <c r="F156" s="6" t="s">
         <v>641</v>
       </c>
       <c r="G156" s="1" t="s">
@@ -7676,7 +7682,7 @@
         <v>12</v>
       </c>
       <c r="I156" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.3">
@@ -7695,7 +7701,7 @@
       <c r="E157" s="1">
         <v>20251700408</v>
       </c>
-      <c r="F157" s="2" t="s">
+      <c r="F157" s="6" t="s">
         <v>645</v>
       </c>
       <c r="G157" s="1" t="s">
@@ -7705,7 +7711,7 @@
         <v>12</v>
       </c>
       <c r="I157" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="158" spans="1:9" x14ac:dyDescent="0.3">
@@ -7724,7 +7730,7 @@
       <c r="E158" s="1">
         <v>20241700014</v>
       </c>
-      <c r="F158" s="2" t="s">
+      <c r="F158" s="6" t="s">
         <v>649</v>
       </c>
       <c r="G158" s="1" t="s">
@@ -7734,7 +7740,7 @@
         <v>12</v>
       </c>
       <c r="I158" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.3">
@@ -7753,7 +7759,7 @@
       <c r="E159" s="1">
         <v>20251700766</v>
       </c>
-      <c r="F159" s="2" t="s">
+      <c r="F159" s="6" t="s">
         <v>653</v>
       </c>
       <c r="G159" s="1" t="s">
@@ -7763,7 +7769,7 @@
         <v>12</v>
       </c>
       <c r="I159" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="160" spans="1:9" x14ac:dyDescent="0.3">
@@ -7782,7 +7788,7 @@
       <c r="E160" s="1">
         <v>2021170551</v>
       </c>
-      <c r="F160" s="2" t="s">
+      <c r="F160" s="6" t="s">
         <v>657</v>
       </c>
       <c r="G160" s="1" t="s">
@@ -7792,7 +7798,7 @@
         <v>126</v>
       </c>
       <c r="I160" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="161" spans="1:9" x14ac:dyDescent="0.3">
@@ -7811,7 +7817,7 @@
       <c r="E161" s="1">
         <v>2022170350</v>
       </c>
-      <c r="F161" s="2" t="s">
+      <c r="F161" s="6" t="s">
         <v>661</v>
       </c>
       <c r="G161" s="1" t="s">
@@ -7821,7 +7827,7 @@
         <v>48</v>
       </c>
       <c r="I161" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="162" spans="1:9" x14ac:dyDescent="0.3">
@@ -7840,7 +7846,7 @@
       <c r="E162" s="1">
         <v>20241700581</v>
       </c>
-      <c r="F162" s="2" t="s">
+      <c r="F162" s="6" t="s">
         <v>665</v>
       </c>
       <c r="G162" s="1" t="s">
@@ -7850,7 +7856,7 @@
         <v>12</v>
       </c>
       <c r="I162" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="163" spans="1:9" x14ac:dyDescent="0.3">
@@ -7869,7 +7875,7 @@
       <c r="E163" s="1">
         <v>20251700101</v>
       </c>
-      <c r="F163" s="2" t="s">
+      <c r="F163" s="6" t="s">
         <v>669</v>
       </c>
       <c r="G163" s="1" t="s">
@@ -7879,7 +7885,7 @@
         <v>12</v>
       </c>
       <c r="I163" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="164" spans="1:9" x14ac:dyDescent="0.3">
@@ -7898,7 +7904,7 @@
       <c r="E164" s="1">
         <v>20241700141</v>
       </c>
-      <c r="F164" s="2" t="s">
+      <c r="F164" s="6" t="s">
         <v>673</v>
       </c>
       <c r="G164" s="1" t="s">
@@ -7908,7 +7914,7 @@
         <v>12</v>
       </c>
       <c r="I164" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="165" spans="1:9" x14ac:dyDescent="0.3">
@@ -7927,7 +7933,7 @@
       <c r="E165" s="1">
         <v>20241701175</v>
       </c>
-      <c r="F165" s="2" t="s">
+      <c r="F165" s="6" t="s">
         <v>677</v>
       </c>
       <c r="G165" s="1" t="s">
@@ -7937,7 +7943,7 @@
         <v>12</v>
       </c>
       <c r="I165" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="166" spans="1:9" x14ac:dyDescent="0.3">
@@ -7956,7 +7962,7 @@
       <c r="E166" s="1">
         <v>20241701614</v>
       </c>
-      <c r="F166" s="2" t="s">
+      <c r="F166" s="6" t="s">
         <v>681</v>
       </c>
       <c r="G166" s="1" t="s">
@@ -7966,7 +7972,7 @@
         <v>207</v>
       </c>
       <c r="I166" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="167" spans="1:9" x14ac:dyDescent="0.3">
@@ -7985,7 +7991,7 @@
       <c r="E167" s="1">
         <v>20251700290</v>
       </c>
-      <c r="F167" s="2" t="s">
+      <c r="F167" s="6" t="s">
         <v>685</v>
       </c>
       <c r="G167" s="1" t="s">
@@ -7995,7 +8001,7 @@
         <v>12</v>
       </c>
       <c r="I167" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="168" spans="1:9" x14ac:dyDescent="0.3">
@@ -8014,7 +8020,7 @@
       <c r="E168" s="1">
         <v>20231700231</v>
       </c>
-      <c r="F168" s="2" t="s">
+      <c r="F168" s="6" t="s">
         <v>689</v>
       </c>
       <c r="G168" s="1" t="s">
@@ -8024,7 +8030,7 @@
         <v>207</v>
       </c>
       <c r="I168" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="169" spans="1:9" x14ac:dyDescent="0.3">
@@ -8043,7 +8049,7 @@
       <c r="E169" s="1">
         <v>20241700761</v>
       </c>
-      <c r="F169" s="2" t="s">
+      <c r="F169" s="6" t="s">
         <v>693</v>
       </c>
       <c r="G169" s="1" t="s">
@@ -8053,7 +8059,7 @@
         <v>12</v>
       </c>
       <c r="I169" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="170" spans="1:9" x14ac:dyDescent="0.3">
@@ -8072,7 +8078,7 @@
       <c r="E170" s="1">
         <v>20251700360</v>
       </c>
-      <c r="F170" s="2" t="s">
+      <c r="F170" s="6" t="s">
         <v>697</v>
       </c>
       <c r="G170" s="1" t="s">
@@ -8082,7 +8088,7 @@
         <v>12</v>
       </c>
       <c r="I170" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="171" spans="1:9" x14ac:dyDescent="0.3">
@@ -8101,7 +8107,7 @@
       <c r="E171" s="1">
         <v>20251701139</v>
       </c>
-      <c r="F171" s="2" t="s">
+      <c r="F171" s="6" t="s">
         <v>701</v>
       </c>
       <c r="G171" s="1" t="s">
@@ -8111,7 +8117,7 @@
         <v>12</v>
       </c>
       <c r="I171" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="172" spans="1:9" x14ac:dyDescent="0.3">
@@ -8130,7 +8136,7 @@
       <c r="E172" s="1">
         <v>2022170372</v>
       </c>
-      <c r="F172" s="2" t="s">
+      <c r="F172" s="6" t="s">
         <v>705</v>
       </c>
       <c r="G172" s="1" t="s">
@@ -8140,7 +8146,7 @@
         <v>48</v>
       </c>
       <c r="I172" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="173" spans="1:9" x14ac:dyDescent="0.3">
@@ -8159,7 +8165,7 @@
       <c r="E173" s="1">
         <v>20241700185</v>
       </c>
-      <c r="F173" s="2" t="s">
+      <c r="F173" s="6" t="s">
         <v>709</v>
       </c>
       <c r="G173" s="1" t="s">
@@ -8169,7 +8175,7 @@
         <v>12</v>
       </c>
       <c r="I173" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="174" spans="1:9" x14ac:dyDescent="0.3">
@@ -8188,7 +8194,7 @@
       <c r="E174" s="1">
         <v>20251701144</v>
       </c>
-      <c r="F174" s="2" t="s">
+      <c r="F174" s="6" t="s">
         <v>713</v>
       </c>
       <c r="G174" s="1" t="s">
@@ -8198,7 +8204,7 @@
         <v>12</v>
       </c>
       <c r="I174" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.3">
@@ -8217,7 +8223,7 @@
       <c r="E175" s="1">
         <v>2023170730</v>
       </c>
-      <c r="F175" s="2" t="s">
+      <c r="F175" s="6" t="s">
         <v>717</v>
       </c>
       <c r="G175" s="1" t="s">
@@ -8227,7 +8233,7 @@
         <v>377</v>
       </c>
       <c r="I175" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.3">
@@ -8246,7 +8252,7 @@
       <c r="E176" s="1">
         <v>20241700910</v>
       </c>
-      <c r="F176" s="2" t="s">
+      <c r="F176" s="6" t="s">
         <v>721</v>
       </c>
       <c r="G176" s="1" t="s">
@@ -8256,7 +8262,7 @@
         <v>12</v>
       </c>
       <c r="I176" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.3">
@@ -8275,7 +8281,7 @@
       <c r="E177" s="1">
         <v>20251701023</v>
       </c>
-      <c r="F177" s="2" t="s">
+      <c r="F177" s="6" t="s">
         <v>725</v>
       </c>
       <c r="G177" s="1" t="s">
@@ -8285,7 +8291,7 @@
         <v>12</v>
       </c>
       <c r="I177" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="178" spans="1:9" x14ac:dyDescent="0.3">
@@ -8304,7 +8310,7 @@
       <c r="E178" s="1">
         <v>20241701617</v>
       </c>
-      <c r="F178" s="2" t="s">
+      <c r="F178" s="6" t="s">
         <v>729</v>
       </c>
       <c r="G178" s="1" t="s">
@@ -8314,7 +8320,7 @@
         <v>207</v>
       </c>
       <c r="I178" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.3">
@@ -8333,7 +8339,7 @@
       <c r="E179" s="1">
         <v>20241701611</v>
       </c>
-      <c r="F179" s="2" t="s">
+      <c r="F179" s="6" t="s">
         <v>733</v>
       </c>
       <c r="G179" s="1" t="s">
@@ -8343,7 +8349,7 @@
         <v>207</v>
       </c>
       <c r="I179" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="180" spans="1:9" x14ac:dyDescent="0.3">
@@ -8362,7 +8368,7 @@
       <c r="E180" s="1">
         <v>20241700483</v>
       </c>
-      <c r="F180" s="2" t="s">
+      <c r="F180" s="6" t="s">
         <v>737</v>
       </c>
       <c r="G180" s="1" t="s">
@@ -8372,7 +8378,7 @@
         <v>12</v>
       </c>
       <c r="I180" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="181" spans="1:9" x14ac:dyDescent="0.3">
@@ -8391,7 +8397,7 @@
       <c r="E181" s="1">
         <v>2022170261</v>
       </c>
-      <c r="F181" s="2" t="s">
+      <c r="F181" s="6" t="s">
         <v>741</v>
       </c>
       <c r="G181" s="1" t="s">
@@ -8401,7 +8407,7 @@
         <v>48</v>
       </c>
       <c r="I181" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="182" spans="1:9" x14ac:dyDescent="0.3">
@@ -8420,7 +8426,7 @@
       <c r="E182" s="1">
         <v>20241700848</v>
       </c>
-      <c r="F182" s="2" t="s">
+      <c r="F182" s="6" t="s">
         <v>745</v>
       </c>
       <c r="G182" s="1" t="s">
@@ -8430,7 +8436,7 @@
         <v>12</v>
       </c>
       <c r="I182" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="183" spans="1:9" x14ac:dyDescent="0.3">
@@ -8449,7 +8455,7 @@
       <c r="E183" s="1">
         <v>20241700799</v>
       </c>
-      <c r="F183" s="2" t="s">
+      <c r="F183" s="6" t="s">
         <v>749</v>
       </c>
       <c r="G183" s="1" t="s">
@@ -8459,7 +8465,7 @@
         <v>12</v>
       </c>
       <c r="I183" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="184" spans="1:9" x14ac:dyDescent="0.3">
@@ -8478,7 +8484,7 @@
       <c r="E184" s="1">
         <v>20241700741</v>
       </c>
-      <c r="F184" s="2" t="s">
+      <c r="F184" s="6" t="s">
         <v>753</v>
       </c>
       <c r="G184" s="1" t="s">
@@ -8488,7 +8494,7 @@
         <v>12</v>
       </c>
       <c r="I184" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.3">
@@ -8507,7 +8513,7 @@
       <c r="E185" s="1">
         <v>20241700733</v>
       </c>
-      <c r="F185" s="2" t="s">
+      <c r="F185" s="6" t="s">
         <v>757</v>
       </c>
       <c r="G185" s="1" t="s">
@@ -8517,7 +8523,7 @@
         <v>12</v>
       </c>
       <c r="I185" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="186" spans="1:9" x14ac:dyDescent="0.3">
@@ -8536,7 +8542,7 @@
       <c r="E186" s="1">
         <v>20241700967</v>
       </c>
-      <c r="F186" s="2" t="s">
+      <c r="F186" s="6" t="s">
         <v>761</v>
       </c>
       <c r="G186" s="1" t="s">
@@ -8546,7 +8552,7 @@
         <v>12</v>
       </c>
       <c r="I186" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="187" spans="1:9" x14ac:dyDescent="0.3">
@@ -8565,7 +8571,7 @@
       <c r="E187" s="1">
         <v>20241701557</v>
       </c>
-      <c r="F187" s="2" t="s">
+      <c r="F187" s="6" t="s">
         <v>765</v>
       </c>
       <c r="G187" s="1" t="s">
@@ -8575,7 +8581,7 @@
         <v>402</v>
       </c>
       <c r="I187" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="188" spans="1:9" x14ac:dyDescent="0.3">
@@ -8594,7 +8600,7 @@
       <c r="E188" s="1">
         <v>20241700290</v>
       </c>
-      <c r="F188" s="2" t="s">
+      <c r="F188" s="6" t="s">
         <v>769</v>
       </c>
       <c r="G188" s="1" t="s">
@@ -8604,7 +8610,7 @@
         <v>12</v>
       </c>
       <c r="I188" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="189" spans="1:9" x14ac:dyDescent="0.3">
@@ -8623,7 +8629,7 @@
       <c r="E189" s="1">
         <v>2022170358</v>
       </c>
-      <c r="F189" s="2" t="s">
+      <c r="F189" s="6" t="s">
         <v>773</v>
       </c>
       <c r="G189" s="1" t="s">
@@ -8633,7 +8639,7 @@
         <v>31</v>
       </c>
       <c r="I189" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="190" spans="1:9" x14ac:dyDescent="0.3">
@@ -8652,7 +8658,7 @@
       <c r="E190" s="1">
         <v>20251700975</v>
       </c>
-      <c r="F190" s="2" t="s">
+      <c r="F190" s="6" t="s">
         <v>777</v>
       </c>
       <c r="G190" s="1" t="s">
@@ -8662,7 +8668,7 @@
         <v>12</v>
       </c>
       <c r="I190" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="191" spans="1:9" x14ac:dyDescent="0.3">
@@ -8681,7 +8687,7 @@
       <c r="E191" s="1">
         <v>20251701092</v>
       </c>
-      <c r="F191" s="2" t="s">
+      <c r="F191" s="6" t="s">
         <v>781</v>
       </c>
       <c r="G191" s="1" t="s">
@@ -8691,7 +8697,7 @@
         <v>12</v>
       </c>
       <c r="I191" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="192" spans="1:9" x14ac:dyDescent="0.3">
@@ -8710,7 +8716,7 @@
       <c r="E192" s="1">
         <v>20251700579</v>
       </c>
-      <c r="F192" s="2" t="s">
+      <c r="F192" s="6" t="s">
         <v>785</v>
       </c>
       <c r="G192" s="1" t="s">
@@ -8720,7 +8726,7 @@
         <v>12</v>
       </c>
       <c r="I192" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="193" spans="1:9" x14ac:dyDescent="0.3">
@@ -8739,7 +8745,7 @@
       <c r="E193" s="1">
         <v>20231700104</v>
       </c>
-      <c r="F193" s="2" t="s">
+      <c r="F193" s="6" t="s">
         <v>789</v>
       </c>
       <c r="G193" s="1" t="s">
@@ -8749,7 +8755,7 @@
         <v>113</v>
       </c>
       <c r="I193" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="194" spans="1:9" x14ac:dyDescent="0.3">
@@ -8768,7 +8774,7 @@
       <c r="E194" s="1">
         <v>20251700504</v>
       </c>
-      <c r="F194" s="1" t="s">
+      <c r="F194" s="3" t="s">
         <v>793</v>
       </c>
       <c r="G194" s="1" t="s">
@@ -8778,7 +8784,7 @@
         <v>12</v>
       </c>
       <c r="I194" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="195" spans="1:9" x14ac:dyDescent="0.3">
@@ -8797,7 +8803,7 @@
       <c r="E195" s="1">
         <v>20251701133</v>
       </c>
-      <c r="F195" s="1" t="s">
+      <c r="F195" s="3" t="s">
         <v>797</v>
       </c>
       <c r="G195" s="1" t="s">
@@ -8807,7 +8813,7 @@
         <v>12</v>
       </c>
       <c r="I195" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="196" spans="1:9" x14ac:dyDescent="0.3">
@@ -8826,7 +8832,7 @@
       <c r="E196" s="1">
         <v>20241700560</v>
       </c>
-      <c r="F196" s="1" t="s">
+      <c r="F196" s="3" t="s">
         <v>801</v>
       </c>
       <c r="G196" s="1" t="s">
@@ -8836,7 +8842,7 @@
         <v>12</v>
       </c>
       <c r="I196" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="197" spans="1:9" x14ac:dyDescent="0.3">
@@ -8855,7 +8861,7 @@
       <c r="E197" s="1">
         <v>20241701173</v>
       </c>
-      <c r="F197" s="1" t="s">
+      <c r="F197" s="3" t="s">
         <v>805</v>
       </c>
       <c r="G197" s="1" t="s">
@@ -8865,7 +8871,7 @@
         <v>12</v>
       </c>
       <c r="I197" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="198" spans="1:9" x14ac:dyDescent="0.3">
@@ -8884,7 +8890,7 @@
       <c r="E198" s="1">
         <v>20241700628</v>
       </c>
-      <c r="F198" s="1" t="s">
+      <c r="F198" s="3" t="s">
         <v>809</v>
       </c>
       <c r="G198" s="1" t="s">
@@ -8894,36 +8900,40 @@
         <v>12</v>
       </c>
       <c r="I198" s="1" t="s">
-        <v>905</v>
+        <v>904</v>
       </c>
     </row>
     <row r="199" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A199" s="1"/>
+      <c r="A199" s="1">
+        <v>198</v>
+      </c>
       <c r="B199" s="1"/>
       <c r="C199" s="1" t="s">
         <v>810</v>
       </c>
-      <c r="D199" s="3" t="s">
+      <c r="D199" s="2" t="s">
         <v>811</v>
       </c>
       <c r="E199" s="1">
         <v>20241700183</v>
       </c>
-      <c r="F199" s="4" t="s">
+      <c r="F199" s="3" t="s">
         <v>812</v>
       </c>
       <c r="G199" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="H199" s="5" t="s">
+      <c r="H199" s="4" t="s">
         <v>813</v>
       </c>
-      <c r="I199" s="5" t="s">
+      <c r="I199" s="4" t="s">
         <v>814</v>
       </c>
     </row>
     <row r="200" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A200" s="1"/>
+      <c r="A200" s="1">
+        <v>199</v>
+      </c>
       <c r="B200" s="1"/>
       <c r="C200" s="1" t="s">
         <v>815</v>
@@ -8934,21 +8944,23 @@
       <c r="E200" s="1">
         <v>20241700872</v>
       </c>
-      <c r="F200" s="4" t="s">
+      <c r="F200" s="3" t="s">
         <v>817</v>
       </c>
       <c r="G200" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="H200" s="5" t="s">
+      <c r="H200" s="4" t="s">
         <v>813</v>
       </c>
-      <c r="I200" s="5" t="s">
+      <c r="I200" s="4" t="s">
         <v>814</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A201" s="1"/>
+      <c r="A201" s="1">
+        <v>200</v>
+      </c>
       <c r="B201" s="1"/>
       <c r="C201" s="1" t="s">
         <v>818</v>
@@ -8959,7 +8971,7 @@
       <c r="E201" s="1" t="s">
         <v>820</v>
       </c>
-      <c r="F201" s="4" t="s">
+      <c r="F201" s="3" t="s">
         <v>821</v>
       </c>
       <c r="G201" s="1" t="s">
@@ -8968,12 +8980,14 @@
       <c r="H201" s="1" t="s">
         <v>822</v>
       </c>
-      <c r="I201" s="5" t="s">
+      <c r="I201" s="4" t="s">
         <v>823</v>
       </c>
     </row>
     <row r="202" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A202" s="1"/>
+      <c r="A202" s="1">
+        <v>201</v>
+      </c>
       <c r="B202" s="1"/>
       <c r="C202" s="1" t="s">
         <v>824</v>
@@ -8984,7 +8998,7 @@
       <c r="E202" s="1" t="s">
         <v>826</v>
       </c>
-      <c r="F202" s="4" t="s">
+      <c r="F202" s="3" t="s">
         <v>827</v>
       </c>
       <c r="G202" s="1" t="s">
@@ -8993,12 +9007,14 @@
       <c r="H202" s="1" t="s">
         <v>828</v>
       </c>
-      <c r="I202" s="5" t="s">
+      <c r="I202" s="4" t="s">
         <v>823</v>
       </c>
     </row>
     <row r="203" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A203" s="1"/>
+      <c r="A203" s="1">
+        <v>202</v>
+      </c>
       <c r="B203" s="1"/>
       <c r="C203" s="1" t="s">
         <v>829</v>
@@ -9009,7 +9025,7 @@
       <c r="E203" s="1" t="s">
         <v>831</v>
       </c>
-      <c r="F203" s="4" t="s">
+      <c r="F203" s="3" t="s">
         <v>832</v>
       </c>
       <c r="G203" s="1" t="s">
@@ -9018,12 +9034,14 @@
       <c r="H203" s="1" t="s">
         <v>822</v>
       </c>
-      <c r="I203" s="5" t="s">
+      <c r="I203" s="4" t="s">
         <v>823</v>
       </c>
     </row>
     <row r="204" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A204" s="1"/>
+      <c r="A204" s="1">
+        <v>203</v>
+      </c>
       <c r="B204" s="1"/>
       <c r="C204" s="1" t="s">
         <v>833</v>
@@ -9034,7 +9052,7 @@
       <c r="E204" s="1" t="s">
         <v>835</v>
       </c>
-      <c r="F204" s="4" t="s">
+      <c r="F204" s="3" t="s">
         <v>836</v>
       </c>
       <c r="G204" s="1" t="s">
@@ -9043,12 +9061,14 @@
       <c r="H204" s="1" t="s">
         <v>822</v>
       </c>
-      <c r="I204" s="5" t="s">
+      <c r="I204" s="4" t="s">
         <v>823</v>
       </c>
     </row>
     <row r="205" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A205" s="1"/>
+      <c r="A205" s="1">
+        <v>204</v>
+      </c>
       <c r="B205" s="1"/>
       <c r="C205" s="1" t="s">
         <v>837</v>
@@ -9059,7 +9079,7 @@
       <c r="E205" s="1" t="s">
         <v>839</v>
       </c>
-      <c r="F205" s="4" t="s">
+      <c r="F205" s="3" t="s">
         <v>840</v>
       </c>
       <c r="G205" s="1" t="s">
@@ -9068,12 +9088,14 @@
       <c r="H205" s="1" t="s">
         <v>822</v>
       </c>
-      <c r="I205" s="5" t="s">
+      <c r="I205" s="4" t="s">
         <v>841</v>
       </c>
     </row>
     <row r="206" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A206" s="1"/>
+      <c r="A206" s="1">
+        <v>205</v>
+      </c>
       <c r="B206" s="1"/>
       <c r="C206" s="1" t="s">
         <v>842</v>
@@ -9084,7 +9106,7 @@
       <c r="E206" s="1" t="s">
         <v>844</v>
       </c>
-      <c r="F206" s="4" t="s">
+      <c r="F206" s="3" t="s">
         <v>845</v>
       </c>
       <c r="G206" s="1" t="s">
@@ -9093,12 +9115,14 @@
       <c r="H206" s="1" t="s">
         <v>822</v>
       </c>
-      <c r="I206" s="5" t="s">
+      <c r="I206" s="4" t="s">
         <v>841</v>
       </c>
     </row>
     <row r="207" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A207" s="1"/>
+      <c r="A207" s="1">
+        <v>206</v>
+      </c>
       <c r="B207" s="1"/>
       <c r="C207" s="1" t="s">
         <v>846</v>
@@ -9109,7 +9133,7 @@
       <c r="E207" s="1" t="s">
         <v>848</v>
       </c>
-      <c r="F207" s="4" t="s">
+      <c r="F207" s="3" t="s">
         <v>849</v>
       </c>
       <c r="G207" s="1" t="s">
@@ -9118,12 +9142,14 @@
       <c r="H207" s="1" t="s">
         <v>813</v>
       </c>
-      <c r="I207" s="5" t="s">
+      <c r="I207" s="4" t="s">
         <v>841</v>
       </c>
     </row>
     <row r="208" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A208" s="1"/>
+      <c r="A208" s="1">
+        <v>207</v>
+      </c>
       <c r="B208" s="1"/>
       <c r="C208" s="1" t="s">
         <v>850</v>
@@ -9134,7 +9160,7 @@
       <c r="E208" s="1" t="s">
         <v>852</v>
       </c>
-      <c r="F208" s="4" t="s">
+      <c r="F208" s="3" t="s">
         <v>853</v>
       </c>
       <c r="G208" s="1" t="s">
@@ -9143,12 +9169,14 @@
       <c r="H208" s="1" t="s">
         <v>813</v>
       </c>
-      <c r="I208" s="5" t="s">
+      <c r="I208" s="4" t="s">
         <v>841</v>
       </c>
     </row>
     <row r="209" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A209" s="1"/>
+      <c r="A209" s="1">
+        <v>208</v>
+      </c>
       <c r="B209" s="1"/>
       <c r="C209" s="1" t="s">
         <v>854</v>
@@ -9159,7 +9187,7 @@
       <c r="E209" s="1" t="s">
         <v>856</v>
       </c>
-      <c r="F209" s="4" t="s">
+      <c r="F209" s="3" t="s">
         <v>857</v>
       </c>
       <c r="G209" s="1" t="s">
@@ -9168,12 +9196,14 @@
       <c r="H209" s="1" t="s">
         <v>822</v>
       </c>
-      <c r="I209" s="5" t="s">
+      <c r="I209" s="4" t="s">
         <v>841</v>
       </c>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A210" s="1"/>
+      <c r="A210" s="1">
+        <v>209</v>
+      </c>
       <c r="B210" s="1"/>
       <c r="C210" s="1" t="s">
         <v>858</v>
@@ -9184,7 +9214,7 @@
       <c r="E210" s="1" t="s">
         <v>860</v>
       </c>
-      <c r="F210" s="4" t="s">
+      <c r="F210" s="3" t="s">
         <v>861</v>
       </c>
       <c r="G210" s="1" t="s">
@@ -9193,12 +9223,14 @@
       <c r="H210" s="1" t="s">
         <v>822</v>
       </c>
-      <c r="I210" s="5" t="s">
+      <c r="I210" s="4" t="s">
         <v>841</v>
       </c>
     </row>
     <row r="211" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A211" s="1"/>
+      <c r="A211" s="1">
+        <v>210</v>
+      </c>
       <c r="B211" s="1"/>
       <c r="C211" s="1" t="s">
         <v>862</v>
@@ -9209,7 +9241,7 @@
       <c r="E211" s="1" t="s">
         <v>864</v>
       </c>
-      <c r="F211" s="4" t="s">
+      <c r="F211" s="3" t="s">
         <v>865</v>
       </c>
       <c r="G211" s="1" t="s">
@@ -9218,12 +9250,14 @@
       <c r="H211" s="1" t="s">
         <v>866</v>
       </c>
-      <c r="I211" s="5" t="s">
+      <c r="I211" s="4" t="s">
         <v>814</v>
       </c>
     </row>
     <row r="212" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A212" s="1"/>
+      <c r="A212" s="1">
+        <v>211</v>
+      </c>
       <c r="B212" s="1"/>
       <c r="C212" s="1" t="s">
         <v>867</v>
@@ -9234,7 +9268,7 @@
       <c r="E212" s="1">
         <v>20231700519</v>
       </c>
-      <c r="F212" s="4" t="s">
+      <c r="F212" s="3" t="s">
         <v>869</v>
       </c>
       <c r="G212" s="1" t="s">
@@ -9243,12 +9277,14 @@
       <c r="H212" s="1" t="s">
         <v>633</v>
       </c>
-      <c r="I212" s="5" t="s">
+      <c r="I212" s="4" t="s">
         <v>814</v>
       </c>
     </row>
     <row r="213" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A213" s="1"/>
+      <c r="A213" s="1">
+        <v>212</v>
+      </c>
       <c r="B213" s="1"/>
       <c r="C213" s="1" t="s">
         <v>870</v>
@@ -9259,7 +9295,7 @@
       <c r="E213" s="1" t="s">
         <v>872</v>
       </c>
-      <c r="F213" s="4" t="s">
+      <c r="F213" s="3" t="s">
         <v>873</v>
       </c>
       <c r="G213" s="1" t="s">
@@ -9268,12 +9304,14 @@
       <c r="H213" s="1" t="s">
         <v>813</v>
       </c>
-      <c r="I213" s="5" t="s">
+      <c r="I213" s="4" t="s">
         <v>814</v>
       </c>
     </row>
     <row r="214" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A214" s="1"/>
+      <c r="A214" s="1">
+        <v>213</v>
+      </c>
       <c r="B214" s="1"/>
       <c r="C214" s="1" t="s">
         <v>874</v>
@@ -9284,7 +9322,7 @@
       <c r="E214" s="1" t="s">
         <v>876</v>
       </c>
-      <c r="F214" s="4" t="s">
+      <c r="F214" s="3" t="s">
         <v>877</v>
       </c>
       <c r="G214" s="1" t="s">
@@ -9293,12 +9331,14 @@
       <c r="H214" s="1" t="s">
         <v>813</v>
       </c>
-      <c r="I214" s="5" t="s">
+      <c r="I214" s="4" t="s">
         <v>814</v>
       </c>
     </row>
     <row r="215" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A215" s="1"/>
+      <c r="A215" s="1">
+        <v>214</v>
+      </c>
       <c r="B215" s="1"/>
       <c r="C215" s="1" t="s">
         <v>878</v>
@@ -9309,7 +9349,7 @@
       <c r="E215" s="1" t="s">
         <v>880</v>
       </c>
-      <c r="F215" s="4" t="s">
+      <c r="F215" s="3" t="s">
         <v>881</v>
       </c>
       <c r="G215" s="1" t="s">
@@ -9318,12 +9358,14 @@
       <c r="H215" s="1" t="s">
         <v>813</v>
       </c>
-      <c r="I215" s="5" t="s">
+      <c r="I215" s="4" t="s">
         <v>814</v>
       </c>
     </row>
     <row r="216" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A216" s="1"/>
+      <c r="A216" s="1">
+        <v>215</v>
+      </c>
       <c r="B216" s="1"/>
       <c r="C216" s="1" t="s">
         <v>882</v>
@@ -9334,7 +9376,7 @@
       <c r="E216" s="1" t="s">
         <v>884</v>
       </c>
-      <c r="F216" s="4" t="s">
+      <c r="F216" s="3" t="s">
         <v>885</v>
       </c>
       <c r="G216" s="1" t="s">
@@ -9343,23 +9385,25 @@
       <c r="H216" s="1" t="s">
         <v>813</v>
       </c>
-      <c r="I216" s="5" t="s">
-        <v>814</v>
+      <c r="I216" s="4" t="s">
+        <v>823</v>
       </c>
     </row>
     <row r="217" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A217" s="1"/>
+      <c r="A217" s="1">
+        <v>216</v>
+      </c>
       <c r="B217" s="1"/>
       <c r="C217" s="1" t="s">
         <v>886</v>
       </c>
-      <c r="D217" s="3" t="s">
+      <c r="D217" s="2" t="s">
         <v>887</v>
       </c>
       <c r="E217" s="1" t="s">
         <v>888</v>
       </c>
-      <c r="F217" s="4" t="s">
+      <c r="F217" s="3" t="s">
         <v>889</v>
       </c>
       <c r="G217" s="1" t="s">
@@ -9368,23 +9412,25 @@
       <c r="H217" s="1" t="s">
         <v>866</v>
       </c>
-      <c r="I217" s="5" t="s">
+      <c r="I217" s="4" t="s">
         <v>814</v>
       </c>
     </row>
     <row r="218" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A218" s="1"/>
+      <c r="A218" s="1">
+        <v>217</v>
+      </c>
       <c r="B218" s="1"/>
       <c r="C218" s="1" t="s">
         <v>890</v>
       </c>
-      <c r="D218" s="3" t="s">
+      <c r="D218" s="2" t="s">
         <v>891</v>
       </c>
       <c r="E218" s="1" t="s">
         <v>892</v>
       </c>
-      <c r="F218" s="4" t="s">
+      <c r="F218" s="3" t="s">
         <v>893</v>
       </c>
       <c r="G218" s="1" t="s">
@@ -9393,135 +9439,161 @@
       <c r="H218" s="1" t="s">
         <v>813</v>
       </c>
-      <c r="I218" s="5" t="s">
+      <c r="I218" s="4" t="s">
         <v>814</v>
       </c>
     </row>
     <row r="219" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A219" s="1"/>
+      <c r="A219" s="1">
+        <v>219</v>
+      </c>
       <c r="B219" s="1"/>
-      <c r="C219" s="5" t="s">
+      <c r="C219" s="4" t="s">
+        <v>895</v>
+      </c>
+      <c r="D219" s="4" t="s">
+        <v>896</v>
+      </c>
+      <c r="E219" s="4">
+        <v>20251700722</v>
+      </c>
+      <c r="F219" s="5" t="s">
+        <v>897</v>
+      </c>
+      <c r="G219" s="4" t="s">
         <v>894</v>
       </c>
-      <c r="D219" s="6" t="s">
-        <v>883</v>
-      </c>
-      <c r="E219" s="5">
-        <v>20251700393</v>
-      </c>
-      <c r="F219" s="7" t="s">
-        <v>885</v>
-      </c>
-      <c r="G219" s="5" t="s">
-        <v>895</v>
-      </c>
-      <c r="H219" s="5" t="s">
+      <c r="H219" s="4" t="s">
         <v>813</v>
       </c>
-      <c r="I219" s="5" t="s">
+      <c r="I219" s="4" t="s">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="220" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A220" s="1">
+        <v>220</v>
+      </c>
+      <c r="B220" s="1"/>
+      <c r="C220" s="1" t="s">
+        <v>898</v>
+      </c>
+      <c r="D220" s="1" t="s">
+        <v>899</v>
+      </c>
+      <c r="E220" s="1">
+        <v>2023170630</v>
+      </c>
+      <c r="F220" s="3" t="s">
+        <v>900</v>
+      </c>
+      <c r="G220" s="1" t="s">
+        <v>901</v>
+      </c>
+      <c r="H220" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="I220" s="4" t="s">
         <v>841</v>
       </c>
     </row>
-    <row r="220" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A220" s="1"/>
-      <c r="B220" s="1"/>
-      <c r="C220" s="5" t="s">
-        <v>896</v>
-      </c>
-      <c r="D220" s="5" t="s">
-        <v>897</v>
-      </c>
-      <c r="E220" s="5">
-        <v>20251700722</v>
-      </c>
-      <c r="F220" s="7" t="s">
-        <v>898</v>
-      </c>
-      <c r="G220" s="5" t="s">
-        <v>895</v>
-      </c>
-      <c r="H220" s="5" t="s">
-        <v>813</v>
-      </c>
-      <c r="I220" s="5" t="s">
-        <v>814</v>
-      </c>
-    </row>
     <row r="221" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A221" s="1"/>
+      <c r="A221" s="1">
+        <v>222</v>
+      </c>
       <c r="B221" s="1"/>
       <c r="C221" s="1" t="s">
-        <v>899</v>
-      </c>
-      <c r="D221" s="1" t="s">
-        <v>900</v>
+        <v>906</v>
+      </c>
+      <c r="D221" s="2" t="s">
+        <v>910</v>
       </c>
       <c r="E221" s="1">
-        <v>2023170630</v>
-      </c>
-      <c r="F221" s="4" t="s">
+        <v>2023170714</v>
+      </c>
+      <c r="F221" s="3" t="s">
+        <v>915</v>
+      </c>
+      <c r="G221" s="1" t="s">
         <v>901</v>
       </c>
-      <c r="G221" s="1" t="s">
-        <v>902</v>
-      </c>
       <c r="H221" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="I221" s="5" t="s">
-        <v>841</v>
+        <v>866</v>
+      </c>
+      <c r="I221" s="4" t="s">
+        <v>905</v>
       </c>
     </row>
     <row r="222" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A222" s="1">
+        <v>223</v>
+      </c>
+      <c r="B222" s="1"/>
       <c r="C222" s="1" t="s">
-        <v>906</v>
-      </c>
-      <c r="D222" s="8" t="s">
         <v>907</v>
       </c>
+      <c r="D222" s="2" t="s">
+        <v>911</v>
+      </c>
       <c r="E222" s="1">
-        <v>2023170570</v>
-      </c>
-      <c r="F222" s="4" t="s">
+        <v>2022170578</v>
+      </c>
+      <c r="F222" s="3" t="s">
+        <v>913</v>
+      </c>
+      <c r="G222" s="1" t="s">
+        <v>916</v>
+      </c>
+      <c r="H222" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="I222" s="4" t="s">
+        <v>823</v>
+      </c>
+    </row>
+    <row r="223" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A223" s="1">
+        <v>224</v>
+      </c>
+      <c r="B223" s="1"/>
+      <c r="C223" s="1" t="s">
         <v>908</v>
       </c>
-      <c r="G222" s="1" t="s">
-        <v>902</v>
-      </c>
-      <c r="H222" s="1" t="s">
+      <c r="D223" s="2" t="s">
+        <v>912</v>
+      </c>
+      <c r="E223" s="1">
+        <v>2023170573</v>
+      </c>
+      <c r="F223" s="3" t="s">
+        <v>914</v>
+      </c>
+      <c r="G223" s="1" t="s">
+        <v>901</v>
+      </c>
+      <c r="H223" s="1" t="s">
         <v>866</v>
       </c>
-      <c r="I222" s="5" t="s">
+      <c r="I223" s="4" t="s">
         <v>909</v>
       </c>
     </row>
-    <row r="223" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="C223" s="1" t="s">
-        <v>910</v>
-      </c>
-      <c r="I223" s="5" t="s">
-        <v>909</v>
-      </c>
-    </row>
     <row r="224" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="C224" s="1" t="s">
-        <v>911</v>
-      </c>
-      <c r="I224" s="5" t="s">
-        <v>823</v>
-      </c>
-    </row>
-    <row r="225" spans="3:9" x14ac:dyDescent="0.3">
-      <c r="C225" s="1" t="s">
-        <v>912</v>
-      </c>
-      <c r="I225" s="5" t="s">
-        <v>913</v>
-      </c>
+      <c r="A224" s="1">
+        <v>225</v>
+      </c>
+      <c r="B224" s="1"/>
+      <c r="C224" s="1"/>
+      <c r="D224" s="1"/>
+      <c r="E224" s="1"/>
+      <c r="F224" s="3"/>
+      <c r="G224" s="1"/>
+      <c r="H224" s="1"/>
+      <c r="I224" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="E1:E295">
+  <conditionalFormatting sqref="E224:E293 E1:E220">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>COUNTIF($F:$F, E1)&gt;1</formula>
     </cfRule>
@@ -9530,8 +9602,9 @@
     <hyperlink ref="D199" r:id="rId1" xr:uid="{07DFA687-492B-4F56-83C7-C75437411F46}"/>
     <hyperlink ref="D218" r:id="rId2" xr:uid="{C9AE0FF3-43B9-461C-8703-0440C05FCB87}"/>
     <hyperlink ref="D217" r:id="rId3" xr:uid="{1537C871-1AE3-43F1-A149-F5E9552895FC}"/>
-    <hyperlink ref="D219" r:id="rId4" xr:uid="{8826757F-1E9F-45FF-A54F-E937E06587D6}"/>
-    <hyperlink ref="D222" r:id="rId5" xr:uid="{811C7B9D-63E5-4FFC-B3AF-05A59466F993}"/>
+    <hyperlink ref="D221" r:id="rId4" xr:uid="{F7884A69-4A0E-429E-BA06-727B89451555}"/>
+    <hyperlink ref="D222" r:id="rId5" xr:uid="{F9E5C2CE-6B37-4ED7-8F55-955B3A60395F}"/>
+    <hyperlink ref="D223" r:id="rId6" xr:uid="{63DF18AE-D025-455A-B8DE-5EC9D24B42E6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>